<commit_message>
Feat: Correção no processo de envio dos emails.
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flytour-my.sharepoint.com/personal/nicolas_cavalcante_flytour_com_br/Documents/Documentos/GitHub/projeto-conciliacao_ebta/logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_2B59D2BFD330D4862FDC2391501518F37CBFF1CF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E96BC22C-3844-4B85-B236-177B4ED9CECF}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_2B59D2BFD3C0D51A49CCE8F1531518F37CBFF40F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FF6E43D-1766-4E7A-9B01-F166F5E1FEAE}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="1050" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>id_execucao</t>
   </si>
@@ -68,6 +68,18 @@
   </si>
   <si>
     <t>Não</t>
+  </si>
+  <si>
+    <t>7f748327-101b-4674-9b1c-c6aca6e24277</t>
+  </si>
+  <si>
+    <t>Sucesso</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>15d5f5bf-9ec5-46ee-869c-3dbd1633ebc5</t>
   </si>
 </sst>
 </file>
@@ -411,12 +423,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.5546875" customWidth="1"/>
-    <col min="3" max="4" width="15.5546875" customWidth="1"/>
-    <col min="5" max="5" width="15.109375" customWidth="1"/>
+    <col min="1" max="1" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" customWidth="1"/>
+    <col min="4" max="5" width="19" customWidth="1"/>
+    <col min="6" max="6" width="24.77734375" customWidth="1"/>
+    <col min="7" max="7" width="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -482,7 +497,7 @@
         <v>14</v>
       </c>
       <c r="B3" s="1">
-        <v>46101.744150012622</v>
+        <v>46101.744150011567</v>
       </c>
       <c r="D3">
         <v>1337</v>
@@ -498,6 +513,58 @@
       </c>
       <c r="H3" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46105.49553414352</v>
+      </c>
+      <c r="D4">
+        <v>1337</v>
+      </c>
+      <c r="E4">
+        <v>634</v>
+      </c>
+      <c r="F4">
+        <v>490</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46105.504587209951</v>
+      </c>
+      <c r="D5">
+        <v>1337</v>
+      </c>
+      <c r="E5">
+        <v>634</v>
+      </c>
+      <c r="F5">
+        <v>490</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Alterações feitas:  Criação da interface com os caminhos dinamicos
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46105.72659389357</v>
+        <v>46105.72659388889</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
@@ -707,6 +707,74 @@
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>796cb36c-84d0-4038-a291-0cabced923f1</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46106.52857400463</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>1337</v>
+      </c>
+      <c r="E9" t="n">
+        <v>635</v>
+      </c>
+      <c r="F9" t="n">
+        <v>489</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>af09102b-88af-46b6-b47a-c93fbcc16f90</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>46106.61111591548</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>1337</v>
+      </c>
+      <c r="E10" t="n">
+        <v>635</v>
+      </c>
+      <c r="F10" t="n">
+        <v>489</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat:Novas bibliotecas incluidas no requirements
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46106.61111591548</v>
+        <v>46106.61111591435</v>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
@@ -775,6 +775,40 @@
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1649c248-fa1b-48ee-98b7-ab9553d634b8</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46107.53537293198</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>1337</v>
+      </c>
+      <c r="E11" t="n">
+        <v>635</v>
+      </c>
+      <c r="F11" t="n">
+        <v>489</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Inclusão de apontamento de erros ao importar arquivo de clientes fora do padrão
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>46107.764147412</v>
+        <v>46107.7641474074</v>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="n">
@@ -979,6 +979,40 @@
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>864afcf5-cd10-4021-b3e0-925393c3ce76</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>46108.38015482599</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>1337</v>
+      </c>
+      <c r="E17" t="n">
+        <v>635</v>
+      </c>
+      <c r="F17" t="n">
+        <v>487</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Novas atualizações feitas
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,42 +433,27 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>arquivo</t>
+          <t>qtd_total</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>qtd_total</t>
+          <t>qtd_corretos</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>qtd_corretos</t>
+          <t>qtd_nao_localizados</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>qtd_nao_localizados</t>
+          <t>status_execucao</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>status_execucao</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
           <t>email_enviado</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>tipo_envio</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>dias_para_corte</t>
         </is>
       </c>
     </row>
@@ -481,32 +466,25 @@
       <c r="B2" s="1" t="n">
         <v>46101.72573665509</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>C:\Users\nicolas.cavalcante\OneDrive - BEFLY TRAVEL\Área de Trabalho\Teste_python\EBTA\PendenciasAereo_20260305-092004.xlsx</t>
-        </is>
+      <c r="C2" t="n">
+        <v>1337</v>
       </c>
       <c r="D2" t="n">
         <v>1337</v>
       </c>
       <c r="E2" t="n">
-        <v>1337</v>
-      </c>
-      <c r="F2" t="n">
         <v>491</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -517,28 +495,25 @@
       <c r="B3" s="1" t="n">
         <v>46101.74415001157</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="n">
+        <v>1337</v>
+      </c>
       <c r="D3" t="n">
-        <v>1337</v>
+        <v>633</v>
       </c>
       <c r="E3" t="n">
-        <v>633</v>
-      </c>
-      <c r="F3" t="n">
         <v>491</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -549,29 +524,24 @@
       <c r="B4" s="1" t="n">
         <v>46105.49553414352</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>1337</v>
+      </c>
       <c r="D4" t="n">
-        <v>1337</v>
+        <v>634</v>
       </c>
       <c r="E4" t="n">
-        <v>634</v>
-      </c>
-      <c r="F4" t="n">
         <v>490</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -583,29 +553,24 @@
       <c r="B5" s="1" t="n">
         <v>46105.50458721065</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="n">
+        <v>1337</v>
+      </c>
       <c r="D5" t="n">
-        <v>1337</v>
+        <v>634</v>
       </c>
       <c r="E5" t="n">
-        <v>634</v>
-      </c>
-      <c r="F5" t="n">
         <v>490</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -617,29 +582,24 @@
       <c r="B6" s="1" t="n">
         <v>46105.64980530093</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="n">
+        <v>1337</v>
+      </c>
       <c r="D6" t="n">
-        <v>1337</v>
+        <v>634</v>
       </c>
       <c r="E6" t="n">
-        <v>634</v>
-      </c>
-      <c r="F6" t="n">
         <v>490</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -651,29 +611,24 @@
       <c r="B7" s="1" t="n">
         <v>46105.7068744213</v>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="n">
+        <v>1337</v>
+      </c>
       <c r="D7" t="n">
-        <v>1337</v>
+        <v>634</v>
       </c>
       <c r="E7" t="n">
-        <v>634</v>
-      </c>
-      <c r="F7" t="n">
         <v>490</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -685,29 +640,24 @@
       <c r="B8" s="1" t="n">
         <v>46105.72659388889</v>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="n">
+        <v>1337</v>
+      </c>
       <c r="D8" t="n">
-        <v>1337</v>
+        <v>634</v>
       </c>
       <c r="E8" t="n">
-        <v>634</v>
-      </c>
-      <c r="F8" t="n">
         <v>490</v>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -719,29 +669,24 @@
       <c r="B9" s="1" t="n">
         <v>46106.52857400463</v>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="n">
+        <v>1337</v>
+      </c>
       <c r="D9" t="n">
-        <v>1337</v>
+        <v>635</v>
       </c>
       <c r="E9" t="n">
-        <v>635</v>
-      </c>
-      <c r="F9" t="n">
         <v>489</v>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -753,29 +698,24 @@
       <c r="B10" s="1" t="n">
         <v>46106.61111591435</v>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="n">
+        <v>1337</v>
+      </c>
       <c r="D10" t="n">
-        <v>1337</v>
+        <v>635</v>
       </c>
       <c r="E10" t="n">
-        <v>635</v>
-      </c>
-      <c r="F10" t="n">
         <v>489</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -787,29 +727,24 @@
       <c r="B11" s="1" t="n">
         <v>46107.53537292824</v>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="n">
+        <v>1337</v>
+      </c>
       <c r="D11" t="n">
-        <v>1337</v>
+        <v>635</v>
       </c>
       <c r="E11" t="n">
-        <v>635</v>
-      </c>
-      <c r="F11" t="n">
         <v>489</v>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -821,29 +756,24 @@
       <c r="B12" s="1" t="n">
         <v>46107.72410099537</v>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="n">
+        <v>1337</v>
+      </c>
       <c r="D12" t="n">
-        <v>1337</v>
+        <v>635</v>
       </c>
       <c r="E12" t="n">
-        <v>635</v>
-      </c>
-      <c r="F12" t="n">
         <v>489</v>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -855,29 +785,24 @@
       <c r="B13" s="1" t="n">
         <v>46107.75169979167</v>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="n">
+        <v>1337</v>
+      </c>
       <c r="D13" t="n">
-        <v>1337</v>
+        <v>635</v>
       </c>
       <c r="E13" t="n">
-        <v>635</v>
-      </c>
-      <c r="F13" t="n">
         <v>489</v>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -889,29 +814,24 @@
       <c r="B14" s="1" t="n">
         <v>46107.75318391203</v>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="n">
+        <v>1337</v>
+      </c>
       <c r="D14" t="n">
-        <v>1337</v>
+        <v>635</v>
       </c>
       <c r="E14" t="n">
-        <v>635</v>
-      </c>
-      <c r="F14" t="n">
         <v>489</v>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -923,29 +843,24 @@
       <c r="B15" s="1" t="n">
         <v>46107.76272480324</v>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="n">
+        <v>1337</v>
+      </c>
       <c r="D15" t="n">
-        <v>1337</v>
+        <v>635</v>
       </c>
       <c r="E15" t="n">
-        <v>635</v>
-      </c>
-      <c r="F15" t="n">
         <v>489</v>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -957,29 +872,24 @@
       <c r="B16" s="1" t="n">
         <v>46107.7641474074</v>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="n">
+        <v>1337</v>
+      </c>
       <c r="D16" t="n">
-        <v>1337</v>
+        <v>635</v>
       </c>
       <c r="E16" t="n">
-        <v>635</v>
-      </c>
-      <c r="F16" t="n">
         <v>489</v>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="n">
-        <v>0</v>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -989,31 +899,345 @@
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>46108.38015482599</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
+        <v>46108.38015482639</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1337</v>
+      </c>
       <c r="D17" t="n">
-        <v>1337</v>
+        <v>635</v>
       </c>
       <c r="E17" t="n">
+        <v>487</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>092004</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>46108.41948178241</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1337</v>
+      </c>
+      <c r="D18" t="n">
         <v>635</v>
       </c>
-      <c r="F17" t="n">
+      <c r="E18" t="n">
         <v>487</v>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Sucesso</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="n">
-        <v>0</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>092004</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>46108.42668966435</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1337</v>
+      </c>
+      <c r="D19" t="n">
+        <v>635</v>
+      </c>
+      <c r="E19" t="n">
+        <v>487</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>46108.42809303241</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>46108.49330347222</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>46108.49732836805</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>46108.49900649305</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>46108.50200325232</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="n">
+        <v>46108.50965956019</v>
+      </c>
+      <c r="C25" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>46108.5224010301</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>46108.52614480324</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>46108.54349105868</v>
+      </c>
+      <c r="C28" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Novas atualizações        Ajustes realizados:
Inclusão de apontamento de erros ao importar arquivo de clientes fora do padrão;
Alteração no layout do fluxo;
Correção no id no log de execução;
Ajuste na lógica do e-mail:
Construção de classificações para os casos de aging corte;
Comparação de casos hj vs ontem;
Reestruturação do corpo do email.
Inclusão da diretoria em cópia quando temos casos inferiores a 0 no aging corte;
Inclusão de um status com classificações no df_não_localizados.
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>46108.54349105868</v>
+        <v>46108.54349105324</v>
       </c>
       <c r="C28" t="n">
         <v>2918</v>
@@ -1235,6 +1235,35 @@
         </is>
       </c>
       <c r="G28" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="n">
+        <v>46108.76424127414</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1023</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
Feat: atualização nas etapas da interface
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="B29" s="1" t="n">
-        <v>46108.76424127414</v>
+        <v>46108.76424127315</v>
       </c>
       <c r="C29" t="n">
         <v>2918</v>
@@ -1264,6 +1264,673 @@
         </is>
       </c>
       <c r="G29" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>46111.6100391088</v>
+      </c>
+      <c r="C30" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="n">
+        <v>46111.61220746528</v>
+      </c>
+      <c r="C31" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="n">
+        <v>46111.61331707176</v>
+      </c>
+      <c r="C32" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="n">
+        <v>46111.61688907407</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="n">
+        <v>46111.62535091435</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E34" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>46111.62897652778</v>
+      </c>
+      <c r="C35" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>46111.63565164352</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E36" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>46111.64350358796</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="n">
+        <v>46111.6626446875</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="n">
+        <v>46111.68665987268</v>
+      </c>
+      <c r="C39" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="n">
+        <v>46111.71419354167</v>
+      </c>
+      <c r="C40" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="n">
+        <v>46111.72252438658</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>46111.72863543982</v>
+      </c>
+      <c r="C42" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="n">
+        <v>46111.73043177083</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="n">
+        <v>46111.73282126158</v>
+      </c>
+      <c r="C44" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>46111.73566465278</v>
+      </c>
+      <c r="C45" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>46111.74317759259</v>
+      </c>
+      <c r="C46" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="n">
+        <v>46111.74475103009</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="n">
+        <v>46111.74552133102</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D48" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="n">
+        <v>46111.74670564815</v>
+      </c>
+      <c r="C49" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="n">
+        <v>46111.75431741899</v>
+      </c>
+      <c r="C50" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D50" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="n">
+        <v>46111.7563621875</v>
+      </c>
+      <c r="C51" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D51" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="n">
+        <v>46111.76060545169</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D52" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
Feat: Atualizações na interface
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1914,7 +1914,7 @@
         </is>
       </c>
       <c r="B52" s="1" t="n">
-        <v>46111.76060545169</v>
+        <v>46111.76060545139</v>
       </c>
       <c r="C52" t="n">
         <v>2918</v>
@@ -1931,6 +1931,325 @@
         </is>
       </c>
       <c r="G52" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="n">
+        <v>46112.41025875</v>
+      </c>
+      <c r="C53" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="n">
+        <v>46112.41942771991</v>
+      </c>
+      <c r="C54" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="n">
+        <v>46112.42704112268</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="n">
+        <v>46112.43096738426</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="n">
+        <v>46112.43348075231</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>46112.43673467592</v>
+      </c>
+      <c r="C58" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E58" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="n">
+        <v>46112.4497774537</v>
+      </c>
+      <c r="C59" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E59" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="n">
+        <v>46112.4535002199</v>
+      </c>
+      <c r="C60" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D60" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E60" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="n">
+        <v>46112.45566394676</v>
+      </c>
+      <c r="C61" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E61" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>175004</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>46112.46075384259</v>
+      </c>
+      <c r="C62" t="n">
+        <v>2918</v>
+      </c>
+      <c r="D62" t="n">
+        <v>1353</v>
+      </c>
+      <c r="E62" t="n">
+        <v>1020</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="n">
+        <v>46112.66317863045</v>
+      </c>
+      <c r="C63" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D63" t="n">
+        <v>929</v>
+      </c>
+      <c r="E63" t="n">
+        <v>1038</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
feat: Data fechamento incluida
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="B63" s="1" t="n">
-        <v>46112.66317863045</v>
+        <v>46112.66317863426</v>
       </c>
       <c r="C63" t="n">
         <v>2483</v>
@@ -2250,6 +2250,64 @@
         </is>
       </c>
       <c r="G63" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>46113.74308824074</v>
+      </c>
+      <c r="C64" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D64" t="n">
+        <v>932</v>
+      </c>
+      <c r="E64" t="n">
+        <v>1035</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>46113.74703734838</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D65" t="n">
+        <v>932</v>
+      </c>
+      <c r="E65" t="n">
+        <v>1035</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
Feat: Alterações na busca de dados
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="B73" s="1" t="n">
-        <v>46118.75285546029</v>
+        <v>46118.75285546296</v>
       </c>
       <c r="C73" t="n">
         <v>2483</v>
@@ -2540,6 +2540,267 @@
         </is>
       </c>
       <c r="G73" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B74" s="1" t="n">
+        <v>46119.39567476852</v>
+      </c>
+      <c r="C74" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1553</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B75" s="1" t="n">
+        <v>46119.43846362268</v>
+      </c>
+      <c r="C75" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D75" t="n">
+        <v>1004</v>
+      </c>
+      <c r="E75" t="n">
+        <v>930</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B76" s="1" t="n">
+        <v>46119.45169223379</v>
+      </c>
+      <c r="C76" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D76" t="n">
+        <v>1553</v>
+      </c>
+      <c r="E76" t="n">
+        <v>930</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B77" s="1" t="n">
+        <v>46119.53283692129</v>
+      </c>
+      <c r="C77" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D77" t="n">
+        <v>1553</v>
+      </c>
+      <c r="E77" t="n">
+        <v>930</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B78" s="1" t="n">
+        <v>46119.62383178241</v>
+      </c>
+      <c r="C78" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D78" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B79" s="1" t="n">
+        <v>46119.67646815972</v>
+      </c>
+      <c r="C79" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B80" s="1" t="n">
+        <v>46119.71791038194</v>
+      </c>
+      <c r="C80" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B81" s="1" t="n">
+        <v>46119.72231275463</v>
+      </c>
+      <c r="C81" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D81" t="n">
+        <v>589</v>
+      </c>
+      <c r="E81" t="n">
+        <v>930</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B82" s="1" t="n">
+        <v>46119.7537994379</v>
+      </c>
+      <c r="C82" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D82" t="n">
+        <v>589</v>
+      </c>
+      <c r="E82" t="n">
+        <v>930</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
Feat: alterações e validações nos matchings
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2784,7 +2784,7 @@
         </is>
       </c>
       <c r="B82" s="1" t="n">
-        <v>46119.7537994379</v>
+        <v>46119.75379943287</v>
       </c>
       <c r="C82" t="n">
         <v>2483</v>
@@ -2801,6 +2801,122 @@
         </is>
       </c>
       <c r="G82" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B83" s="1" t="n">
+        <v>46120.39368251157</v>
+      </c>
+      <c r="C83" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D83" t="n">
+        <v>590</v>
+      </c>
+      <c r="E83" t="n">
+        <v>924</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B84" s="1" t="n">
+        <v>46120.39890835648</v>
+      </c>
+      <c r="C84" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D84" t="n">
+        <v>590</v>
+      </c>
+      <c r="E84" t="n">
+        <v>924</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B85" s="1" t="n">
+        <v>46120.40575290509</v>
+      </c>
+      <c r="C85" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D85" t="n">
+        <v>590</v>
+      </c>
+      <c r="E85" t="n">
+        <v>924</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B86" s="1" t="n">
+        <v>46120.67720973374</v>
+      </c>
+      <c r="C86" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D86" t="n">
+        <v>590</v>
+      </c>
+      <c r="E86" t="n">
+        <v>924</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
feat: alteração de lib e alteração no layout do arquivo final que sobe ao bradesco
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2900,7 +2900,7 @@
         </is>
       </c>
       <c r="B86" s="1" t="n">
-        <v>46120.67720973374</v>
+        <v>46120.6772097338</v>
       </c>
       <c r="C86" t="n">
         <v>2483</v>
@@ -2917,6 +2917,528 @@
         </is>
       </c>
       <c r="G86" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B87" s="1" t="n">
+        <v>46121.38523392361</v>
+      </c>
+      <c r="C87" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D87" t="n">
+        <v>591</v>
+      </c>
+      <c r="E87" t="n">
+        <v>923</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B88" s="1" t="n">
+        <v>46121.53076859954</v>
+      </c>
+      <c r="C88" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D88" t="n">
+        <v>591</v>
+      </c>
+      <c r="E88" t="n">
+        <v>923</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B89" s="1" t="n">
+        <v>46121.54319725694</v>
+      </c>
+      <c r="C89" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D89" t="n">
+        <v>591</v>
+      </c>
+      <c r="E89" t="n">
+        <v>923</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B90" s="1" t="n">
+        <v>46121.55113340278</v>
+      </c>
+      <c r="C90" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D90" t="n">
+        <v>591</v>
+      </c>
+      <c r="E90" t="n">
+        <v>923</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B91" s="1" t="n">
+        <v>46121.55784666667</v>
+      </c>
+      <c r="C91" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D91" t="n">
+        <v>591</v>
+      </c>
+      <c r="E91" t="n">
+        <v>923</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B92" s="1" t="n">
+        <v>46121.56269762731</v>
+      </c>
+      <c r="C92" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D92" t="n">
+        <v>591</v>
+      </c>
+      <c r="E92" t="n">
+        <v>923</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B93" s="1" t="n">
+        <v>46121.56827375</v>
+      </c>
+      <c r="C93" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D93" t="n">
+        <v>591</v>
+      </c>
+      <c r="E93" t="n">
+        <v>923</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B94" s="1" t="n">
+        <v>46121.6673628588</v>
+      </c>
+      <c r="C94" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D94" t="n">
+        <v>591</v>
+      </c>
+      <c r="E94" t="n">
+        <v>923</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B95" s="1" t="n">
+        <v>46121.66909810185</v>
+      </c>
+      <c r="C95" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D95" t="n">
+        <v>591</v>
+      </c>
+      <c r="E95" t="n">
+        <v>923</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B96" s="1" t="n">
+        <v>46121.67244798611</v>
+      </c>
+      <c r="C96" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D96" t="n">
+        <v>591</v>
+      </c>
+      <c r="E96" t="n">
+        <v>923</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B97" s="1" t="n">
+        <v>46121.67419420139</v>
+      </c>
+      <c r="C97" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D97" t="n">
+        <v>591</v>
+      </c>
+      <c r="E97" t="n">
+        <v>923</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B98" s="1" t="n">
+        <v>46121.67719439815</v>
+      </c>
+      <c r="C98" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D98" t="n">
+        <v>591</v>
+      </c>
+      <c r="E98" t="n">
+        <v>923</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B99" s="1" t="n">
+        <v>46121.68645496527</v>
+      </c>
+      <c r="C99" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D99" t="n">
+        <v>591</v>
+      </c>
+      <c r="E99" t="n">
+        <v>923</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B100" s="1" t="n">
+        <v>46121.68913951389</v>
+      </c>
+      <c r="C100" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D100" t="n">
+        <v>591</v>
+      </c>
+      <c r="E100" t="n">
+        <v>923</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B101" s="1" t="n">
+        <v>46121.7127384375</v>
+      </c>
+      <c r="C101" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D101" t="n">
+        <v>591</v>
+      </c>
+      <c r="E101" t="n">
+        <v>923</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B102" s="1" t="n">
+        <v>46121.72267989584</v>
+      </c>
+      <c r="C102" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D102" t="n">
+        <v>591</v>
+      </c>
+      <c r="E102" t="n">
+        <v>923</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B103" s="1" t="n">
+        <v>46121.72666157407</v>
+      </c>
+      <c r="C103" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D103" t="n">
+        <v>591</v>
+      </c>
+      <c r="E103" t="n">
+        <v>923</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="n">
+        <v>46121.73305842547</v>
+      </c>
+      <c r="C104" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D104" t="n">
+        <v>591</v>
+      </c>
+      <c r="E104" t="n">
+        <v>923</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
Feat: Alteração na lógica de envio de emails para operação e diretoria, baseando-se em um novo calculo de dias restantes. Criação de exceções para tratar possíveis erros durante o processamento
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G105"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3451,7 +3451,7 @@
         </is>
       </c>
       <c r="B105" s="1" t="n">
-        <v>46121.76233723714</v>
+        <v>46121.7623372338</v>
       </c>
       <c r="C105" t="n">
         <v>2483</v>
@@ -3468,6 +3468,151 @@
         </is>
       </c>
       <c r="G105" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="n">
+        <v>46122.406395625</v>
+      </c>
+      <c r="C106" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D106" t="n">
+        <v>591</v>
+      </c>
+      <c r="E106" t="n">
+        <v>923</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="n">
+        <v>46122.47005061342</v>
+      </c>
+      <c r="C107" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D107" t="n">
+        <v>591</v>
+      </c>
+      <c r="E107" t="n">
+        <v>923</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="n">
+        <v>46122.47625121528</v>
+      </c>
+      <c r="C108" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D108" t="n">
+        <v>591</v>
+      </c>
+      <c r="E108" t="n">
+        <v>923</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="n">
+        <v>46122.48558318287</v>
+      </c>
+      <c r="C109" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D109" t="n">
+        <v>591</v>
+      </c>
+      <c r="E109" t="n">
+        <v>923</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B110" s="1" t="n">
+        <v>46122.5204621664</v>
+      </c>
+      <c r="C110" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D110" t="n">
+        <v>591</v>
+      </c>
+      <c r="E110" t="n">
+        <v>923</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
Feat: Novo arquivo de_para incluido, porém sem utilização. Inclusão da qtde de casos não localizados no corpo do e-mail.
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3596,7 +3596,7 @@
         </is>
       </c>
       <c r="B110" s="1" t="n">
-        <v>46122.5204621664</v>
+        <v>46122.52046216435</v>
       </c>
       <c r="C110" t="n">
         <v>2483</v>
@@ -3613,6 +3613,325 @@
         </is>
       </c>
       <c r="G110" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B111" s="1" t="n">
+        <v>46122.61061143519</v>
+      </c>
+      <c r="C111" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D111" t="n">
+        <v>591</v>
+      </c>
+      <c r="E111" t="n">
+        <v>923</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B112" s="1" t="n">
+        <v>46122.61777961806</v>
+      </c>
+      <c r="C112" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D112" t="n">
+        <v>591</v>
+      </c>
+      <c r="E112" t="n">
+        <v>923</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B113" s="1" t="n">
+        <v>46122.62062868055</v>
+      </c>
+      <c r="C113" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D113" t="n">
+        <v>591</v>
+      </c>
+      <c r="E113" t="n">
+        <v>923</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="n">
+        <v>46122.62380298611</v>
+      </c>
+      <c r="C114" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D114" t="n">
+        <v>591</v>
+      </c>
+      <c r="E114" t="n">
+        <v>923</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B115" s="1" t="n">
+        <v>46122.63134145833</v>
+      </c>
+      <c r="C115" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D115" t="n">
+        <v>591</v>
+      </c>
+      <c r="E115" t="n">
+        <v>923</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B116" s="1" t="n">
+        <v>46122.63718284723</v>
+      </c>
+      <c r="C116" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D116" t="n">
+        <v>591</v>
+      </c>
+      <c r="E116" t="n">
+        <v>923</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B117" s="1" t="n">
+        <v>46122.63842409723</v>
+      </c>
+      <c r="C117" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D117" t="n">
+        <v>591</v>
+      </c>
+      <c r="E117" t="n">
+        <v>923</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B118" s="1" t="n">
+        <v>46122.65452885417</v>
+      </c>
+      <c r="C118" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D118" t="n">
+        <v>591</v>
+      </c>
+      <c r="E118" t="n">
+        <v>923</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B119" s="1" t="n">
+        <v>46122.65676549768</v>
+      </c>
+      <c r="C119" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D119" t="n">
+        <v>591</v>
+      </c>
+      <c r="E119" t="n">
+        <v>923</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B120" s="1" t="n">
+        <v>46122.69943885416</v>
+      </c>
+      <c r="C120" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D120" t="n">
+        <v>591</v>
+      </c>
+      <c r="E120" t="n">
+        <v>923</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B121" s="1" t="n">
+        <v>46122.70952173382</v>
+      </c>
+      <c r="C121" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D121" t="n">
+        <v>591</v>
+      </c>
+      <c r="E121" t="n">
+        <v>923</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
Feat: Alteração na lógica de preenchimento utilizando depara de mascara do banco x base do cliente
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="B121" s="1" t="n">
-        <v>46122.70952173382</v>
+        <v>46122.70952173611</v>
       </c>
       <c r="C121" t="n">
         <v>2483</v>
@@ -3932,6 +3932,93 @@
         </is>
       </c>
       <c r="G121" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B122" s="1" t="n">
+        <v>46125.6990255787</v>
+      </c>
+      <c r="C122" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D122" t="n">
+        <v>591</v>
+      </c>
+      <c r="E122" t="n">
+        <v>921</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B123" s="1" t="n">
+        <v>46125.71044626158</v>
+      </c>
+      <c r="C123" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D123" t="n">
+        <v>592</v>
+      </c>
+      <c r="E123" t="n">
+        <v>921</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B124" s="1" t="n">
+        <v>46125.72842457903</v>
+      </c>
+      <c r="C124" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D124" t="n">
+        <v>567</v>
+      </c>
+      <c r="E124" t="n">
+        <v>967</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>

</xml_diff>

<commit_message>
Inclusão de novos arquivos de log + inicio de criaçaõ de nova chave
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G139"/>
+  <dimension ref="A1:I160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,6 +456,16 @@
           <t>email_enviado</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>qtd_correto</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>qtd_nao_localizado</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -485,6 +495,8 @@
           <t>NAO</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -514,6 +526,8 @@
           <t>Não</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -543,6 +557,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -572,6 +588,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -601,6 +619,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -630,6 +650,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -659,6 +681,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -688,6 +712,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -717,6 +743,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -746,6 +774,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -775,6 +805,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -804,6 +836,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -833,6 +867,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -862,6 +898,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -891,6 +929,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -920,6 +960,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -949,6 +991,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -978,6 +1022,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1007,6 +1053,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1036,6 +1084,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1065,6 +1115,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1094,6 +1146,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1123,6 +1177,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1152,6 +1208,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1181,6 +1239,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1210,6 +1270,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1239,6 +1301,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1268,6 +1332,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1297,6 +1363,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1326,6 +1394,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1355,6 +1425,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1384,6 +1456,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1413,6 +1487,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1442,6 +1518,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1471,6 +1549,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1500,6 +1580,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1529,6 +1611,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1558,6 +1642,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1587,6 +1673,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1616,6 +1704,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1645,6 +1735,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1674,6 +1766,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1703,6 +1797,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1732,6 +1828,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1761,6 +1859,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1790,6 +1890,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1819,6 +1921,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1848,6 +1952,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1877,6 +1983,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1906,6 +2014,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1935,6 +2045,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1964,6 +2076,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1993,6 +2107,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2022,6 +2138,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2051,6 +2169,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2080,6 +2200,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2109,6 +2231,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2138,6 +2262,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2167,6 +2293,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2196,6 +2324,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2225,6 +2355,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2254,6 +2386,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2283,6 +2417,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2312,6 +2448,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2341,6 +2479,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2370,6 +2510,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2399,6 +2541,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2428,6 +2572,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2457,6 +2603,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2486,6 +2634,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2515,6 +2665,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2544,6 +2696,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2573,6 +2727,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2602,6 +2758,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2631,6 +2789,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2660,6 +2820,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2689,6 +2851,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2718,6 +2882,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2747,6 +2913,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2776,6 +2944,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2805,6 +2975,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2834,6 +3006,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2863,6 +3037,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2892,6 +3068,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2921,6 +3099,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2950,6 +3130,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2979,6 +3161,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3008,6 +3192,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3037,6 +3223,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3066,6 +3254,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3095,6 +3285,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3124,6 +3316,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3153,6 +3347,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3182,6 +3378,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3211,6 +3409,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3240,6 +3440,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3269,6 +3471,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3298,6 +3502,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3327,6 +3533,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3356,6 +3564,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3385,6 +3595,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3414,6 +3626,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3443,6 +3657,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3472,6 +3688,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3501,6 +3719,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3530,6 +3750,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3559,6 +3781,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3588,6 +3812,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3617,6 +3843,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3646,6 +3874,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3675,6 +3905,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3704,6 +3936,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3733,6 +3967,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3762,6 +3998,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3791,6 +4029,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3820,6 +4060,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3849,6 +4091,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3878,6 +4122,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3907,6 +4153,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3936,6 +4184,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3965,6 +4215,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3994,6 +4246,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4023,6 +4277,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4052,6 +4308,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4081,6 +4339,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4110,6 +4370,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4139,6 +4401,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4168,6 +4432,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4197,6 +4463,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4226,6 +4494,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4255,6 +4525,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4284,6 +4556,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4313,6 +4587,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4342,6 +4618,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4371,6 +4649,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4400,6 +4680,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4429,6 +4711,8 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4437,7 +4721,7 @@
         </is>
       </c>
       <c r="B139" s="1" t="n">
-        <v>46127.74703119617</v>
+        <v>46127.74703119213</v>
       </c>
       <c r="C139" t="n">
         <v>2483</v>
@@ -4457,6 +4741,651 @@
         <is>
           <t>Sim</t>
         </is>
+      </c>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B140" s="1" t="n">
+        <v>46128.49012506945</v>
+      </c>
+      <c r="C140" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D140" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E140" t="n">
+        <v>923</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B141" s="1" t="n">
+        <v>46128.49821149305</v>
+      </c>
+      <c r="C141" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D141" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E141" t="n">
+        <v>923</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B142" s="1" t="n">
+        <v>46128.50918100694</v>
+      </c>
+      <c r="C142" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D142" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E142" t="n">
+        <v>923</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B143" s="1" t="n">
+        <v>46128.51407899305</v>
+      </c>
+      <c r="C143" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D143" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E143" t="n">
+        <v>923</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B144" s="1" t="n">
+        <v>46128.52490581018</v>
+      </c>
+      <c r="C144" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D144" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E144" t="n">
+        <v>923</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B145" s="1" t="n">
+        <v>46128.54265914352</v>
+      </c>
+      <c r="C145" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D145" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E145" t="n">
+        <v>923</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B146" s="1" t="n">
+        <v>46128.60701623843</v>
+      </c>
+      <c r="C146" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D146" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E146" t="n">
+        <v>923</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B147" s="1" t="n">
+        <v>46128.60996971065</v>
+      </c>
+      <c r="C147" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D147" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E147" t="n">
+        <v>923</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B148" s="1" t="n">
+        <v>46128.62062979167</v>
+      </c>
+      <c r="C148" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D148" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E148" t="n">
+        <v>923</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B149" s="1" t="n">
+        <v>46128.63043313658</v>
+      </c>
+      <c r="C149" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D149" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E149" t="n">
+        <v>923</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B150" s="1" t="n">
+        <v>46128.63363145833</v>
+      </c>
+      <c r="C150" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D150" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E150" t="n">
+        <v>923</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B151" s="1" t="n">
+        <v>46128.63707028935</v>
+      </c>
+      <c r="C151" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D151" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E151" t="n">
+        <v>923</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B152" s="1" t="n">
+        <v>46128.63898363426</v>
+      </c>
+      <c r="C152" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D152" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E152" t="n">
+        <v>923</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B153" s="1" t="n">
+        <v>46128.64490034722</v>
+      </c>
+      <c r="C153" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D153" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E153" t="n">
+        <v>923</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B154" s="1" t="n">
+        <v>46128.64767024306</v>
+      </c>
+      <c r="C154" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D154" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E154" t="n">
+        <v>923</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B155" s="1" t="n">
+        <v>46128.64953089121</v>
+      </c>
+      <c r="C155" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D155" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E155" t="n">
+        <v>923</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B156" s="1" t="n">
+        <v>46128.6527353588</v>
+      </c>
+      <c r="C156" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D156" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E156" t="n">
+        <v>923</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B157" s="1" t="n">
+        <v>46128.66449248842</v>
+      </c>
+      <c r="C157" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D157" t="n">
+        <v>1078</v>
+      </c>
+      <c r="E157" t="n">
+        <v>923</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B158" s="1" t="n">
+        <v>46128.69853267361</v>
+      </c>
+      <c r="C158" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B159" s="1" t="n">
+        <v>46128.70377894676</v>
+      </c>
+      <c r="C159" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>143005</t>
+        </is>
+      </c>
+      <c r="B160" s="1" t="n">
+        <v>46128.70976169119</v>
+      </c>
+      <c r="C160" t="n">
+        <v>2483</v>
+      </c>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H160" t="n">
+        <v>1078</v>
+      </c>
+      <c r="I160" t="n">
+        <v>923</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Alterações no log definindo um log por celula + cliente e outro por chave de conciliação. Novas regras foram definidas dentro do arquivo main.py e logger.py
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -1,37 +1,79 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flytour-my.sharepoint.com/personal/nicolas_cavalcante_flytour_com_br/Documents/Documentos/GitHub/projeto-conciliacao_ebta/logs/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_2B59D2BFD3A0D8DC5B9A5B90521518F37CBFF177" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81197176-0AFB-4EAF-972A-E28B7BB8E188}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-21720" yWindow="1050" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t>chave</t>
+  </si>
+  <si>
+    <t>ausencia_de_dados</t>
+  </si>
+  <si>
+    <t>qtd_nao_encontrada</t>
+  </si>
+  <si>
+    <t>qtd_encontrada</t>
+  </si>
+  <si>
+    <t>data_execucao</t>
+  </si>
+  <si>
+    <t>Chave Aut + Data + Valor</t>
+  </si>
+  <si>
+    <t>Chave Cartão + Data + Valor</t>
+  </si>
+  <si>
+    <t>Chave Cartão + Data + Valor + Loc Cia</t>
+  </si>
+  <si>
+    <t>Chave Cartão + Valor + Loc Cia</t>
+  </si>
+  <si>
+    <t>Chave Loc Cia + Data + Valor</t>
+  </si>
+  <si>
+    <t>não_match</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -50,81 +92,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -412,134 +395,134 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>chave</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Colunas com ausência de dados</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>qtd_encontrada</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>qtd_nao_encontrada</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>data_execucao</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Chave Aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>49</v>
-      </c>
-      <c r="C2" t="n">
-        <v>248</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>46134.41688997169</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>76</v>
-      </c>
-      <c r="C3" t="n">
-        <v>251</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>46134.41688997169</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Data + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>46134.41688997169</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>65</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>709</v>
+      </c>
+      <c r="E2" s="1">
+        <v>46134.700002180871</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C5" t="n">
-        <v>135</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>46134.41688997169</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Chave Loc Cia + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>307</v>
-      </c>
-      <c r="C6" t="n">
-        <v>428</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>46134.41688997169</v>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>115</v>
+      </c>
+      <c r="E3" s="1">
+        <v>46134.700002180871</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1">
+        <v>46134.700002180871</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>34</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>143</v>
+      </c>
+      <c r="E5" s="1">
+        <v>46134.700002180871</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>42</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>406</v>
+      </c>
+      <c r="E6" s="1">
+        <v>46134.700002180871</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>924</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1">
+        <v>46134.700002180871</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Inclusão do novo arquivo layout.py para organizar a saída dos arquivos, mais ajustes no arquivo de matching
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -843,7 +843,7 @@
         <v>1709</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>46136.7234509621</v>
+        <v>46136.72345096065</v>
       </c>
     </row>
     <row r="23">
@@ -862,7 +862,7 @@
         <v>1157</v>
       </c>
       <c r="E23" s="1" t="n">
-        <v>46136.7234509621</v>
+        <v>46136.72345096065</v>
       </c>
     </row>
     <row r="24">
@@ -881,7 +881,7 @@
         <v>975</v>
       </c>
       <c r="E24" s="1" t="n">
-        <v>46136.7234509621</v>
+        <v>46136.72345096065</v>
       </c>
     </row>
     <row r="25">
@@ -900,7 +900,463 @@
         <v>1160</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>46136.7234509621</v>
+        <v>46136.72345096065</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>774</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1709</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>46139.47897012731</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1156</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>46139.47897012731</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>181</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>974</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>46139.47897012731</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>545</v>
+      </c>
+      <c r="C29" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1159</v>
+      </c>
+      <c r="E29" s="1" t="n">
+        <v>46139.47897012731</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>774</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1709</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>46139.4986769676</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1156</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>46139.4986769676</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>181</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>974</v>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>46139.4986769676</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>545</v>
+      </c>
+      <c r="C33" t="n">
+        <v>5</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1159</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>46139.4986769676</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>774</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1709</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>46139.53418195602</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1156</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>46139.53418195602</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>181</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>974</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>46139.53418195602</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>545</v>
+      </c>
+      <c r="C37" t="n">
+        <v>5</v>
+      </c>
+      <c r="D37" t="n">
+        <v>1159</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>46139.53418195602</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>775</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1708</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>46139.53967067129</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1155</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <v>46139.53967067129</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>181</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>973</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>46139.53967067129</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>545</v>
+      </c>
+      <c r="C41" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1158</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>46139.53967067129</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>775</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1708</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>46139.54689255787</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>3</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1155</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <v>46139.54689255787</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>181</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>973</v>
+      </c>
+      <c r="E44" s="1" t="n">
+        <v>46139.54689255787</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>545</v>
+      </c>
+      <c r="C45" t="n">
+        <v>5</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1158</v>
+      </c>
+      <c r="E45" s="1" t="n">
+        <v>46139.54689255787</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>775</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1708</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <v>46139.61802309471</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1155</v>
+      </c>
+      <c r="E47" s="1" t="n">
+        <v>46139.61802309471</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>181</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>973</v>
+      </c>
+      <c r="E48" s="1" t="n">
+        <v>46139.61802309471</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>545</v>
+      </c>
+      <c r="C49" t="n">
+        <v>5</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1158</v>
+      </c>
+      <c r="E49" s="1" t="n">
+        <v>46139.61802309471</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Ajuste no config e interface para criação do .exe
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1299,7 +1299,7 @@
         <v>1708</v>
       </c>
       <c r="E46" s="1" t="n">
-        <v>46139.61802309471</v>
+        <v>46139.61802309028</v>
       </c>
     </row>
     <row r="47">
@@ -1318,7 +1318,7 @@
         <v>1155</v>
       </c>
       <c r="E47" s="1" t="n">
-        <v>46139.61802309471</v>
+        <v>46139.61802309028</v>
       </c>
     </row>
     <row r="48">
@@ -1337,7 +1337,7 @@
         <v>973</v>
       </c>
       <c r="E48" s="1" t="n">
-        <v>46139.61802309471</v>
+        <v>46139.61802309028</v>
       </c>
     </row>
     <row r="49">
@@ -1356,7 +1356,83 @@
         <v>1158</v>
       </c>
       <c r="E49" s="1" t="n">
-        <v>46139.61802309471</v>
+        <v>46139.61802309028</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>775</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" t="n">
+        <v>1708</v>
+      </c>
+      <c r="E50" s="1" t="n">
+        <v>46139.74981264526</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>3</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" t="n">
+        <v>1155</v>
+      </c>
+      <c r="E51" s="1" t="n">
+        <v>46139.74981264526</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>181</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>973</v>
+      </c>
+      <c r="E52" s="1" t="n">
+        <v>46139.74981264526</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>545</v>
+      </c>
+      <c r="C53" t="n">
+        <v>5</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1158</v>
+      </c>
+      <c r="E53" s="1" t="n">
+        <v>46139.74981264526</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Alteração na interface em andamento
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1375,7 +1375,7 @@
         <v>1708</v>
       </c>
       <c r="E50" s="1" t="n">
-        <v>46139.74981264526</v>
+        <v>46139.74981265047</v>
       </c>
     </row>
     <row r="51">
@@ -1394,7 +1394,7 @@
         <v>1155</v>
       </c>
       <c r="E51" s="1" t="n">
-        <v>46139.74981264526</v>
+        <v>46139.74981265047</v>
       </c>
     </row>
     <row r="52">
@@ -1413,7 +1413,7 @@
         <v>973</v>
       </c>
       <c r="E52" s="1" t="n">
-        <v>46139.74981264526</v>
+        <v>46139.74981265047</v>
       </c>
     </row>
     <row r="53">
@@ -1432,7 +1432,159 @@
         <v>1158</v>
       </c>
       <c r="E53" s="1" t="n">
-        <v>46139.74981264526</v>
+        <v>46139.74981265047</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>776</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1707</v>
+      </c>
+      <c r="E54" s="1" t="n">
+        <v>46140.44566571759</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E55" s="1" t="n">
+        <v>46140.44566571759</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>182</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="n">
+        <v>972</v>
+      </c>
+      <c r="E56" s="1" t="n">
+        <v>46140.44566571759</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>549</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E57" s="1" t="n">
+        <v>46140.44566571759</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>776</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1707</v>
+      </c>
+      <c r="E58" s="1" t="n">
+        <v>46140.6998079621</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E59" s="1" t="n">
+        <v>46140.6998079621</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>182</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" t="n">
+        <v>972</v>
+      </c>
+      <c r="E60" s="1" t="n">
+        <v>46140.6998079621</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>549</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E61" s="1" t="n">
+        <v>46140.6998079621</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Alterações na estrutura da UI saindo de tk.tk para ctk.ctk, otimizando a visualização da interface, além de correções no processamento carregado e imagens apresentadas na visão, ajustes de posição e modelo do container ainda precisam ser realizados
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1831,7 +1831,7 @@
         <v>1707</v>
       </c>
       <c r="E74" s="1" t="n">
-        <v>46141.72050419643</v>
+        <v>46141.72050420139</v>
       </c>
     </row>
     <row r="75">
@@ -1850,7 +1850,7 @@
         <v>1154</v>
       </c>
       <c r="E75" s="1" t="n">
-        <v>46141.72050419643</v>
+        <v>46141.72050420139</v>
       </c>
     </row>
     <row r="76">
@@ -1869,7 +1869,7 @@
         <v>972</v>
       </c>
       <c r="E76" s="1" t="n">
-        <v>46141.72050419643</v>
+        <v>46141.72050420139</v>
       </c>
     </row>
     <row r="77">
@@ -1888,7 +1888,539 @@
         <v>1157</v>
       </c>
       <c r="E77" s="1" t="n">
-        <v>46141.72050419643</v>
+        <v>46141.72050420139</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>776</v>
+      </c>
+      <c r="C78" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" t="n">
+        <v>1707</v>
+      </c>
+      <c r="E78" s="1" t="n">
+        <v>46142.7394778588</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>3</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E79" s="1" t="n">
+        <v>46142.7394778588</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>182</v>
+      </c>
+      <c r="C80" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" t="n">
+        <v>972</v>
+      </c>
+      <c r="E80" s="1" t="n">
+        <v>46142.7394778588</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>549</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E81" s="1" t="n">
+        <v>46142.7394778588</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>776</v>
+      </c>
+      <c r="C82" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" t="n">
+        <v>1707</v>
+      </c>
+      <c r="E82" s="1" t="n">
+        <v>46142.74168386574</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>3</v>
+      </c>
+      <c r="C83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E83" s="1" t="n">
+        <v>46142.74168386574</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>182</v>
+      </c>
+      <c r="C84" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" t="n">
+        <v>972</v>
+      </c>
+      <c r="E84" s="1" t="n">
+        <v>46142.74168386574</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>549</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E85" s="1" t="n">
+        <v>46142.74168386574</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>776</v>
+      </c>
+      <c r="C86" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" t="n">
+        <v>1707</v>
+      </c>
+      <c r="E86" s="1" t="n">
+        <v>46142.75431618056</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>3</v>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E87" s="1" t="n">
+        <v>46142.75431618056</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>182</v>
+      </c>
+      <c r="C88" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" t="n">
+        <v>972</v>
+      </c>
+      <c r="E88" s="1" t="n">
+        <v>46142.75431618056</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>549</v>
+      </c>
+      <c r="C89" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E89" s="1" t="n">
+        <v>46142.75431618056</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>776</v>
+      </c>
+      <c r="C90" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" t="n">
+        <v>1707</v>
+      </c>
+      <c r="E90" s="1" t="n">
+        <v>46142.75646829861</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>3</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E91" s="1" t="n">
+        <v>46142.75646829861</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>182</v>
+      </c>
+      <c r="C92" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" t="n">
+        <v>972</v>
+      </c>
+      <c r="E92" s="1" t="n">
+        <v>46142.75646829861</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>549</v>
+      </c>
+      <c r="C93" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E93" s="1" t="n">
+        <v>46142.75646829861</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>776</v>
+      </c>
+      <c r="C94" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" t="n">
+        <v>1707</v>
+      </c>
+      <c r="E94" s="1" t="n">
+        <v>46142.76001583333</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>3</v>
+      </c>
+      <c r="C95" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E95" s="1" t="n">
+        <v>46142.76001583333</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>182</v>
+      </c>
+      <c r="C96" t="n">
+        <v>0</v>
+      </c>
+      <c r="D96" t="n">
+        <v>972</v>
+      </c>
+      <c r="E96" s="1" t="n">
+        <v>46142.76001583333</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>549</v>
+      </c>
+      <c r="C97" t="n">
+        <v>1</v>
+      </c>
+      <c r="D97" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E97" s="1" t="n">
+        <v>46142.76001583333</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>776</v>
+      </c>
+      <c r="C98" t="n">
+        <v>0</v>
+      </c>
+      <c r="D98" t="n">
+        <v>1707</v>
+      </c>
+      <c r="E98" s="1" t="n">
+        <v>46142.76142811342</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>3</v>
+      </c>
+      <c r="C99" t="n">
+        <v>0</v>
+      </c>
+      <c r="D99" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E99" s="1" t="n">
+        <v>46142.76142811342</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>182</v>
+      </c>
+      <c r="C100" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100" t="n">
+        <v>972</v>
+      </c>
+      <c r="E100" s="1" t="n">
+        <v>46142.76142811342</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>549</v>
+      </c>
+      <c r="C101" t="n">
+        <v>1</v>
+      </c>
+      <c r="D101" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E101" s="1" t="n">
+        <v>46142.76142811342</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>776</v>
+      </c>
+      <c r="C102" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" t="n">
+        <v>1707</v>
+      </c>
+      <c r="E102" s="1" t="n">
+        <v>46142.76646849565</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>3</v>
+      </c>
+      <c r="C103" t="n">
+        <v>0</v>
+      </c>
+      <c r="D103" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E103" s="1" t="n">
+        <v>46142.76646849565</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>182</v>
+      </c>
+      <c r="C104" t="n">
+        <v>0</v>
+      </c>
+      <c r="D104" t="n">
+        <v>972</v>
+      </c>
+      <c r="E104" s="1" t="n">
+        <v>46142.76646849565</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>549</v>
+      </c>
+      <c r="C105" t="n">
+        <v>1</v>
+      </c>
+      <c r="D105" t="n">
+        <v>1157</v>
+      </c>
+      <c r="E105" s="1" t="n">
+        <v>46142.76646849565</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Ajustes no container do processamento realizados. Preenchimento ok; ' layout do banco ok inserindo o nome Pendencias na aba do arquivo final; ' fluxo de email funcional porém ainda sem a base para cruzamento; ' Ajustes na busca de datas do arquivo database.py, ajustando a lógica para puxar mais meses; ' Interface apresenta lentidão em algumas partes de processamento, necessario validar
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E105"/>
+  <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2363,7 +2363,7 @@
         <v>1707</v>
       </c>
       <c r="E102" s="1" t="n">
-        <v>46142.76646849565</v>
+        <v>46142.76646849537</v>
       </c>
     </row>
     <row r="103">
@@ -2382,7 +2382,7 @@
         <v>1154</v>
       </c>
       <c r="E103" s="1" t="n">
-        <v>46142.76646849565</v>
+        <v>46142.76646849537</v>
       </c>
     </row>
     <row r="104">
@@ -2401,7 +2401,7 @@
         <v>972</v>
       </c>
       <c r="E104" s="1" t="n">
-        <v>46142.76646849565</v>
+        <v>46142.76646849537</v>
       </c>
     </row>
     <row r="105">
@@ -2420,7 +2420,463 @@
         <v>1157</v>
       </c>
       <c r="E105" s="1" t="n">
-        <v>46142.76646849565</v>
+        <v>46142.76646849537</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>750</v>
+      </c>
+      <c r="C106" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" t="n">
+        <v>1733</v>
+      </c>
+      <c r="E106" s="1" t="n">
+        <v>46146.40322216435</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>3</v>
+      </c>
+      <c r="C107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E107" s="1" t="n">
+        <v>46146.40322216435</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>171</v>
+      </c>
+      <c r="C108" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" t="n">
+        <v>1029</v>
+      </c>
+      <c r="E108" s="1" t="n">
+        <v>46146.40322216435</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>529</v>
+      </c>
+      <c r="C109" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" t="n">
+        <v>1203</v>
+      </c>
+      <c r="E109" s="1" t="n">
+        <v>46146.40322216435</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>750</v>
+      </c>
+      <c r="C110" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" t="n">
+        <v>1733</v>
+      </c>
+      <c r="E110" s="1" t="n">
+        <v>46146.41637784722</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>3</v>
+      </c>
+      <c r="C111" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E111" s="1" t="n">
+        <v>46146.41637784722</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>171</v>
+      </c>
+      <c r="C112" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" t="n">
+        <v>1029</v>
+      </c>
+      <c r="E112" s="1" t="n">
+        <v>46146.41637784722</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>529</v>
+      </c>
+      <c r="C113" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" t="n">
+        <v>1203</v>
+      </c>
+      <c r="E113" s="1" t="n">
+        <v>46146.41637784722</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>750</v>
+      </c>
+      <c r="C114" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" t="n">
+        <v>1733</v>
+      </c>
+      <c r="E114" s="1" t="n">
+        <v>46146.42939364583</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>3</v>
+      </c>
+      <c r="C115" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E115" s="1" t="n">
+        <v>46146.42939364583</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>171</v>
+      </c>
+      <c r="C116" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" t="n">
+        <v>1029</v>
+      </c>
+      <c r="E116" s="1" t="n">
+        <v>46146.42939364583</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>529</v>
+      </c>
+      <c r="C117" t="n">
+        <v>1</v>
+      </c>
+      <c r="D117" t="n">
+        <v>1203</v>
+      </c>
+      <c r="E117" s="1" t="n">
+        <v>46146.42939364583</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>777</v>
+      </c>
+      <c r="C118" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" t="n">
+        <v>1706</v>
+      </c>
+      <c r="E118" s="1" t="n">
+        <v>46146.4410245949</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>3</v>
+      </c>
+      <c r="C119" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E119" s="1" t="n">
+        <v>46146.4410245949</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>182</v>
+      </c>
+      <c r="C120" t="n">
+        <v>0</v>
+      </c>
+      <c r="D120" t="n">
+        <v>971</v>
+      </c>
+      <c r="E120" s="1" t="n">
+        <v>46146.4410245949</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>549</v>
+      </c>
+      <c r="C121" t="n">
+        <v>1</v>
+      </c>
+      <c r="D121" t="n">
+        <v>1156</v>
+      </c>
+      <c r="E121" s="1" t="n">
+        <v>46146.4410245949</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>777</v>
+      </c>
+      <c r="C122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D122" t="n">
+        <v>1706</v>
+      </c>
+      <c r="E122" s="1" t="n">
+        <v>46146.44760815972</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>3</v>
+      </c>
+      <c r="C123" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E123" s="1" t="n">
+        <v>46146.44760815972</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>182</v>
+      </c>
+      <c r="C124" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" t="n">
+        <v>971</v>
+      </c>
+      <c r="E124" s="1" t="n">
+        <v>46146.44760815972</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>549</v>
+      </c>
+      <c r="C125" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" t="n">
+        <v>1156</v>
+      </c>
+      <c r="E125" s="1" t="n">
+        <v>46146.44760815972</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>777</v>
+      </c>
+      <c r="C126" t="n">
+        <v>0</v>
+      </c>
+      <c r="D126" t="n">
+        <v>1706</v>
+      </c>
+      <c r="E126" s="1" t="n">
+        <v>46146.4687804412</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>3</v>
+      </c>
+      <c r="C127" t="n">
+        <v>0</v>
+      </c>
+      <c r="D127" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E127" s="1" t="n">
+        <v>46146.4687804412</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>182</v>
+      </c>
+      <c r="C128" t="n">
+        <v>0</v>
+      </c>
+      <c r="D128" t="n">
+        <v>971</v>
+      </c>
+      <c r="E128" s="1" t="n">
+        <v>46146.4687804412</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>549</v>
+      </c>
+      <c r="C129" t="n">
+        <v>1</v>
+      </c>
+      <c r="D129" t="n">
+        <v>1156</v>
+      </c>
+      <c r="E129" s="1" t="n">
+        <v>46146.4687804412</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat:Inclusão de nova coluna (autorizacao) como chave, necessário validar os dados que foram incluidos.
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2819,7 +2819,7 @@
         <v>1706</v>
       </c>
       <c r="E126" s="1" t="n">
-        <v>46146.4687804412</v>
+        <v>46146.46878043981</v>
       </c>
     </row>
     <row r="127">
@@ -2838,7 +2838,7 @@
         <v>1153</v>
       </c>
       <c r="E127" s="1" t="n">
-        <v>46146.4687804412</v>
+        <v>46146.46878043981</v>
       </c>
     </row>
     <row r="128">
@@ -2857,7 +2857,7 @@
         <v>971</v>
       </c>
       <c r="E128" s="1" t="n">
-        <v>46146.4687804412</v>
+        <v>46146.46878043981</v>
       </c>
     </row>
     <row r="129">
@@ -2876,7 +2876,197 @@
         <v>1156</v>
       </c>
       <c r="E129" s="1" t="n">
-        <v>46146.4687804412</v>
+        <v>46146.46878043981</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>777</v>
+      </c>
+      <c r="C130" t="n">
+        <v>0</v>
+      </c>
+      <c r="D130" t="n">
+        <v>1706</v>
+      </c>
+      <c r="E130" s="1" t="n">
+        <v>46146.52247116898</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>3</v>
+      </c>
+      <c r="C131" t="n">
+        <v>0</v>
+      </c>
+      <c r="D131" t="n">
+        <v>935</v>
+      </c>
+      <c r="E131" s="1" t="n">
+        <v>46146.52247116898</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>182</v>
+      </c>
+      <c r="C132" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" t="n">
+        <v>753</v>
+      </c>
+      <c r="E132" s="1" t="n">
+        <v>46146.52247116898</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>453</v>
+      </c>
+      <c r="C133" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" t="n">
+        <v>938</v>
+      </c>
+      <c r="E133" s="1" t="n">
+        <v>46146.52247116898</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>312</v>
+      </c>
+      <c r="C134" t="n">
+        <v>3</v>
+      </c>
+      <c r="D134" t="n">
+        <v>1391</v>
+      </c>
+      <c r="E134" s="1" t="n">
+        <v>46146.52247116898</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>777</v>
+      </c>
+      <c r="C135" t="n">
+        <v>0</v>
+      </c>
+      <c r="D135" t="n">
+        <v>1706</v>
+      </c>
+      <c r="E135" s="1" t="n">
+        <v>46146.75858984417</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>3</v>
+      </c>
+      <c r="C136" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" t="n">
+        <v>935</v>
+      </c>
+      <c r="E136" s="1" t="n">
+        <v>46146.75858984417</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>182</v>
+      </c>
+      <c r="C137" t="n">
+        <v>0</v>
+      </c>
+      <c r="D137" t="n">
+        <v>753</v>
+      </c>
+      <c r="E137" s="1" t="n">
+        <v>46146.75858984417</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>453</v>
+      </c>
+      <c r="C138" t="n">
+        <v>0</v>
+      </c>
+      <c r="D138" t="n">
+        <v>938</v>
+      </c>
+      <c r="E138" s="1" t="n">
+        <v>46146.75858984417</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>312</v>
+      </c>
+      <c r="C139" t="n">
+        <v>3</v>
+      </c>
+      <c r="D139" t="n">
+        <v>1391</v>
+      </c>
+      <c r="E139" s="1" t="n">
+        <v>46146.75858984417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajuste na tela de processamento, incluindo nova interface e upload das bases
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4700,7 +4700,7 @@
         <v>1167</v>
       </c>
       <c r="E225" s="1" t="n">
-        <v>46150.63104337532</v>
+        <v>46150.63104337963</v>
       </c>
     </row>
     <row r="226">
@@ -4719,7 +4719,7 @@
         <v>656</v>
       </c>
       <c r="E226" s="1" t="n">
-        <v>46150.63104337532</v>
+        <v>46150.63104337963</v>
       </c>
     </row>
     <row r="227">
@@ -4738,7 +4738,7 @@
         <v>591</v>
       </c>
       <c r="E227" s="1" t="n">
-        <v>46150.63104337532</v>
+        <v>46150.63104337963</v>
       </c>
     </row>
     <row r="228">
@@ -4757,7 +4757,7 @@
         <v>656</v>
       </c>
       <c r="E228" s="1" t="n">
-        <v>46150.63104337532</v>
+        <v>46150.63104337963</v>
       </c>
     </row>
     <row r="229">
@@ -4776,7 +4776,862 @@
         <v>929</v>
       </c>
       <c r="E229" s="1" t="n">
-        <v>46150.63104337532</v>
+        <v>46150.63104337963</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>1497</v>
+      </c>
+      <c r="C230" t="n">
+        <v>0</v>
+      </c>
+      <c r="D230" t="n">
+        <v>1167</v>
+      </c>
+      <c r="E230" s="1" t="n">
+        <v>46150.94713796296</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>0</v>
+      </c>
+      <c r="C231" t="n">
+        <v>0</v>
+      </c>
+      <c r="D231" t="n">
+        <v>656</v>
+      </c>
+      <c r="E231" s="1" t="n">
+        <v>46150.94713796296</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>65</v>
+      </c>
+      <c r="C232" t="n">
+        <v>0</v>
+      </c>
+      <c r="D232" t="n">
+        <v>591</v>
+      </c>
+      <c r="E232" s="1" t="n">
+        <v>46150.94713796296</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>273</v>
+      </c>
+      <c r="C233" t="n">
+        <v>0</v>
+      </c>
+      <c r="D233" t="n">
+        <v>656</v>
+      </c>
+      <c r="E233" s="1" t="n">
+        <v>46150.94713796296</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>238</v>
+      </c>
+      <c r="C234" t="n">
+        <v>0</v>
+      </c>
+      <c r="D234" t="n">
+        <v>929</v>
+      </c>
+      <c r="E234" s="1" t="n">
+        <v>46150.94713796296</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C235" t="n">
+        <v>0</v>
+      </c>
+      <c r="D235" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E235" s="1" t="n">
+        <v>46151.70344542824</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>0</v>
+      </c>
+      <c r="C236" t="n">
+        <v>0</v>
+      </c>
+      <c r="D236" t="n">
+        <v>642</v>
+      </c>
+      <c r="E236" s="1" t="n">
+        <v>46151.70344542824</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>66</v>
+      </c>
+      <c r="C237" t="n">
+        <v>0</v>
+      </c>
+      <c r="D237" t="n">
+        <v>576</v>
+      </c>
+      <c r="E237" s="1" t="n">
+        <v>46151.70344542824</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>274</v>
+      </c>
+      <c r="C238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D238" t="n">
+        <v>642</v>
+      </c>
+      <c r="E238" s="1" t="n">
+        <v>46151.70344542824</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>238</v>
+      </c>
+      <c r="C239" t="n">
+        <v>0</v>
+      </c>
+      <c r="D239" t="n">
+        <v>916</v>
+      </c>
+      <c r="E239" s="1" t="n">
+        <v>46151.70344542824</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C240" t="n">
+        <v>0</v>
+      </c>
+      <c r="D240" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E240" s="1" t="n">
+        <v>46151.756095</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>0</v>
+      </c>
+      <c r="C241" t="n">
+        <v>0</v>
+      </c>
+      <c r="D241" t="n">
+        <v>642</v>
+      </c>
+      <c r="E241" s="1" t="n">
+        <v>46151.756095</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>66</v>
+      </c>
+      <c r="C242" t="n">
+        <v>0</v>
+      </c>
+      <c r="D242" t="n">
+        <v>576</v>
+      </c>
+      <c r="E242" s="1" t="n">
+        <v>46151.756095</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>274</v>
+      </c>
+      <c r="C243" t="n">
+        <v>0</v>
+      </c>
+      <c r="D243" t="n">
+        <v>642</v>
+      </c>
+      <c r="E243" s="1" t="n">
+        <v>46151.756095</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>238</v>
+      </c>
+      <c r="C244" t="n">
+        <v>0</v>
+      </c>
+      <c r="D244" t="n">
+        <v>916</v>
+      </c>
+      <c r="E244" s="1" t="n">
+        <v>46151.756095</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C245" t="n">
+        <v>0</v>
+      </c>
+      <c r="D245" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E245" s="1" t="n">
+        <v>46151.76971546296</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>0</v>
+      </c>
+      <c r="C246" t="n">
+        <v>0</v>
+      </c>
+      <c r="D246" t="n">
+        <v>642</v>
+      </c>
+      <c r="E246" s="1" t="n">
+        <v>46151.76971546296</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>66</v>
+      </c>
+      <c r="C247" t="n">
+        <v>0</v>
+      </c>
+      <c r="D247" t="n">
+        <v>576</v>
+      </c>
+      <c r="E247" s="1" t="n">
+        <v>46151.76971546296</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>274</v>
+      </c>
+      <c r="C248" t="n">
+        <v>0</v>
+      </c>
+      <c r="D248" t="n">
+        <v>642</v>
+      </c>
+      <c r="E248" s="1" t="n">
+        <v>46151.76971546296</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>238</v>
+      </c>
+      <c r="C249" t="n">
+        <v>0</v>
+      </c>
+      <c r="D249" t="n">
+        <v>916</v>
+      </c>
+      <c r="E249" s="1" t="n">
+        <v>46151.76971546296</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C250" t="n">
+        <v>0</v>
+      </c>
+      <c r="D250" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E250" s="1" t="n">
+        <v>46151.77527069444</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>0</v>
+      </c>
+      <c r="C251" t="n">
+        <v>0</v>
+      </c>
+      <c r="D251" t="n">
+        <v>642</v>
+      </c>
+      <c r="E251" s="1" t="n">
+        <v>46151.77527069444</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>66</v>
+      </c>
+      <c r="C252" t="n">
+        <v>0</v>
+      </c>
+      <c r="D252" t="n">
+        <v>576</v>
+      </c>
+      <c r="E252" s="1" t="n">
+        <v>46151.77527069444</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>274</v>
+      </c>
+      <c r="C253" t="n">
+        <v>0</v>
+      </c>
+      <c r="D253" t="n">
+        <v>642</v>
+      </c>
+      <c r="E253" s="1" t="n">
+        <v>46151.77527069444</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>238</v>
+      </c>
+      <c r="C254" t="n">
+        <v>0</v>
+      </c>
+      <c r="D254" t="n">
+        <v>916</v>
+      </c>
+      <c r="E254" s="1" t="n">
+        <v>46151.77527069444</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C255" t="n">
+        <v>0</v>
+      </c>
+      <c r="D255" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E255" s="1" t="n">
+        <v>46151.77715391204</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>0</v>
+      </c>
+      <c r="C256" t="n">
+        <v>0</v>
+      </c>
+      <c r="D256" t="n">
+        <v>642</v>
+      </c>
+      <c r="E256" s="1" t="n">
+        <v>46151.77715391204</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>66</v>
+      </c>
+      <c r="C257" t="n">
+        <v>0</v>
+      </c>
+      <c r="D257" t="n">
+        <v>576</v>
+      </c>
+      <c r="E257" s="1" t="n">
+        <v>46151.77715391204</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>274</v>
+      </c>
+      <c r="C258" t="n">
+        <v>0</v>
+      </c>
+      <c r="D258" t="n">
+        <v>642</v>
+      </c>
+      <c r="E258" s="1" t="n">
+        <v>46151.77715391204</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>238</v>
+      </c>
+      <c r="C259" t="n">
+        <v>0</v>
+      </c>
+      <c r="D259" t="n">
+        <v>916</v>
+      </c>
+      <c r="E259" s="1" t="n">
+        <v>46151.77715391204</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C260" t="n">
+        <v>0</v>
+      </c>
+      <c r="D260" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E260" s="1" t="n">
+        <v>46151.78261204861</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>0</v>
+      </c>
+      <c r="C261" t="n">
+        <v>0</v>
+      </c>
+      <c r="D261" t="n">
+        <v>642</v>
+      </c>
+      <c r="E261" s="1" t="n">
+        <v>46151.78261204861</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>66</v>
+      </c>
+      <c r="C262" t="n">
+        <v>0</v>
+      </c>
+      <c r="D262" t="n">
+        <v>576</v>
+      </c>
+      <c r="E262" s="1" t="n">
+        <v>46151.78261204861</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>274</v>
+      </c>
+      <c r="C263" t="n">
+        <v>0</v>
+      </c>
+      <c r="D263" t="n">
+        <v>642</v>
+      </c>
+      <c r="E263" s="1" t="n">
+        <v>46151.78261204861</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>238</v>
+      </c>
+      <c r="C264" t="n">
+        <v>0</v>
+      </c>
+      <c r="D264" t="n">
+        <v>916</v>
+      </c>
+      <c r="E264" s="1" t="n">
+        <v>46151.78261204861</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C265" t="n">
+        <v>0</v>
+      </c>
+      <c r="D265" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E265" s="1" t="n">
+        <v>46151.78591270834</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>0</v>
+      </c>
+      <c r="C266" t="n">
+        <v>0</v>
+      </c>
+      <c r="D266" t="n">
+        <v>642</v>
+      </c>
+      <c r="E266" s="1" t="n">
+        <v>46151.78591270834</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>66</v>
+      </c>
+      <c r="C267" t="n">
+        <v>0</v>
+      </c>
+      <c r="D267" t="n">
+        <v>576</v>
+      </c>
+      <c r="E267" s="1" t="n">
+        <v>46151.78591270834</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>274</v>
+      </c>
+      <c r="C268" t="n">
+        <v>0</v>
+      </c>
+      <c r="D268" t="n">
+        <v>642</v>
+      </c>
+      <c r="E268" s="1" t="n">
+        <v>46151.78591270834</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>238</v>
+      </c>
+      <c r="C269" t="n">
+        <v>0</v>
+      </c>
+      <c r="D269" t="n">
+        <v>916</v>
+      </c>
+      <c r="E269" s="1" t="n">
+        <v>46151.78591270834</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C270" t="n">
+        <v>0</v>
+      </c>
+      <c r="D270" t="n">
+        <v>1154</v>
+      </c>
+      <c r="E270" s="1" t="n">
+        <v>46151.78753397777</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>0</v>
+      </c>
+      <c r="C271" t="n">
+        <v>0</v>
+      </c>
+      <c r="D271" t="n">
+        <v>642</v>
+      </c>
+      <c r="E271" s="1" t="n">
+        <v>46151.78753397777</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>66</v>
+      </c>
+      <c r="C272" t="n">
+        <v>0</v>
+      </c>
+      <c r="D272" t="n">
+        <v>576</v>
+      </c>
+      <c r="E272" s="1" t="n">
+        <v>46151.78753397777</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>274</v>
+      </c>
+      <c r="C273" t="n">
+        <v>0</v>
+      </c>
+      <c r="D273" t="n">
+        <v>642</v>
+      </c>
+      <c r="E273" s="1" t="n">
+        <v>46151.78753397777</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>238</v>
+      </c>
+      <c r="C274" t="n">
+        <v>0</v>
+      </c>
+      <c r="D274" t="n">
+        <v>916</v>
+      </c>
+      <c r="E274" s="1" t="n">
+        <v>46151.78753397777</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Ajustes no tela_processamento e inclusão de mapeamento de erros no processamento
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E274"/>
+  <dimension ref="A1:E304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5555,7 +5555,7 @@
         <v>1154</v>
       </c>
       <c r="E270" s="1" t="n">
-        <v>46151.78753397777</v>
+        <v>46151.78753398148</v>
       </c>
     </row>
     <row r="271">
@@ -5574,7 +5574,7 @@
         <v>642</v>
       </c>
       <c r="E271" s="1" t="n">
-        <v>46151.78753397777</v>
+        <v>46151.78753398148</v>
       </c>
     </row>
     <row r="272">
@@ -5593,7 +5593,7 @@
         <v>576</v>
       </c>
       <c r="E272" s="1" t="n">
-        <v>46151.78753397777</v>
+        <v>46151.78753398148</v>
       </c>
     </row>
     <row r="273">
@@ -5612,7 +5612,7 @@
         <v>642</v>
       </c>
       <c r="E273" s="1" t="n">
-        <v>46151.78753397777</v>
+        <v>46151.78753398148</v>
       </c>
     </row>
     <row r="274">
@@ -5631,7 +5631,577 @@
         <v>916</v>
       </c>
       <c r="E274" s="1" t="n">
-        <v>46151.78753397777</v>
+        <v>46151.78753398148</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C275" t="n">
+        <v>0</v>
+      </c>
+      <c r="D275" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E275" s="1" t="n">
+        <v>46153.45208097222</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>0</v>
+      </c>
+      <c r="C276" t="n">
+        <v>0</v>
+      </c>
+      <c r="D276" t="n">
+        <v>641</v>
+      </c>
+      <c r="E276" s="1" t="n">
+        <v>46153.45208097222</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>67</v>
+      </c>
+      <c r="C277" t="n">
+        <v>0</v>
+      </c>
+      <c r="D277" t="n">
+        <v>574</v>
+      </c>
+      <c r="E277" s="1" t="n">
+        <v>46153.45208097222</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>274</v>
+      </c>
+      <c r="C278" t="n">
+        <v>0</v>
+      </c>
+      <c r="D278" t="n">
+        <v>641</v>
+      </c>
+      <c r="E278" s="1" t="n">
+        <v>46153.45208097222</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>238</v>
+      </c>
+      <c r="C279" t="n">
+        <v>0</v>
+      </c>
+      <c r="D279" t="n">
+        <v>915</v>
+      </c>
+      <c r="E279" s="1" t="n">
+        <v>46153.45208097222</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C280" t="n">
+        <v>0</v>
+      </c>
+      <c r="D280" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E280" s="1" t="n">
+        <v>46153.4644165625</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>0</v>
+      </c>
+      <c r="C281" t="n">
+        <v>0</v>
+      </c>
+      <c r="D281" t="n">
+        <v>641</v>
+      </c>
+      <c r="E281" s="1" t="n">
+        <v>46153.4644165625</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>67</v>
+      </c>
+      <c r="C282" t="n">
+        <v>0</v>
+      </c>
+      <c r="D282" t="n">
+        <v>574</v>
+      </c>
+      <c r="E282" s="1" t="n">
+        <v>46153.4644165625</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>274</v>
+      </c>
+      <c r="C283" t="n">
+        <v>0</v>
+      </c>
+      <c r="D283" t="n">
+        <v>641</v>
+      </c>
+      <c r="E283" s="1" t="n">
+        <v>46153.4644165625</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>238</v>
+      </c>
+      <c r="C284" t="n">
+        <v>0</v>
+      </c>
+      <c r="D284" t="n">
+        <v>915</v>
+      </c>
+      <c r="E284" s="1" t="n">
+        <v>46153.4644165625</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C285" t="n">
+        <v>0</v>
+      </c>
+      <c r="D285" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E285" s="1" t="n">
+        <v>46153.46758342593</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>0</v>
+      </c>
+      <c r="C286" t="n">
+        <v>0</v>
+      </c>
+      <c r="D286" t="n">
+        <v>641</v>
+      </c>
+      <c r="E286" s="1" t="n">
+        <v>46153.46758342593</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>67</v>
+      </c>
+      <c r="C287" t="n">
+        <v>0</v>
+      </c>
+      <c r="D287" t="n">
+        <v>574</v>
+      </c>
+      <c r="E287" s="1" t="n">
+        <v>46153.46758342593</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>274</v>
+      </c>
+      <c r="C288" t="n">
+        <v>0</v>
+      </c>
+      <c r="D288" t="n">
+        <v>641</v>
+      </c>
+      <c r="E288" s="1" t="n">
+        <v>46153.46758342593</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>238</v>
+      </c>
+      <c r="C289" t="n">
+        <v>0</v>
+      </c>
+      <c r="D289" t="n">
+        <v>915</v>
+      </c>
+      <c r="E289" s="1" t="n">
+        <v>46153.46758342593</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C290" t="n">
+        <v>0</v>
+      </c>
+      <c r="D290" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E290" s="1" t="n">
+        <v>46153.50537142361</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>0</v>
+      </c>
+      <c r="C291" t="n">
+        <v>0</v>
+      </c>
+      <c r="D291" t="n">
+        <v>641</v>
+      </c>
+      <c r="E291" s="1" t="n">
+        <v>46153.50537142361</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>67</v>
+      </c>
+      <c r="C292" t="n">
+        <v>0</v>
+      </c>
+      <c r="D292" t="n">
+        <v>574</v>
+      </c>
+      <c r="E292" s="1" t="n">
+        <v>46153.50537142361</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>274</v>
+      </c>
+      <c r="C293" t="n">
+        <v>0</v>
+      </c>
+      <c r="D293" t="n">
+        <v>641</v>
+      </c>
+      <c r="E293" s="1" t="n">
+        <v>46153.50537142361</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>238</v>
+      </c>
+      <c r="C294" t="n">
+        <v>0</v>
+      </c>
+      <c r="D294" t="n">
+        <v>915</v>
+      </c>
+      <c r="E294" s="1" t="n">
+        <v>46153.50537142361</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C295" t="n">
+        <v>0</v>
+      </c>
+      <c r="D295" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E295" s="1" t="n">
+        <v>46153.50941356482</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>0</v>
+      </c>
+      <c r="C296" t="n">
+        <v>0</v>
+      </c>
+      <c r="D296" t="n">
+        <v>641</v>
+      </c>
+      <c r="E296" s="1" t="n">
+        <v>46153.50941356482</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>67</v>
+      </c>
+      <c r="C297" t="n">
+        <v>0</v>
+      </c>
+      <c r="D297" t="n">
+        <v>574</v>
+      </c>
+      <c r="E297" s="1" t="n">
+        <v>46153.50941356482</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>274</v>
+      </c>
+      <c r="C298" t="n">
+        <v>0</v>
+      </c>
+      <c r="D298" t="n">
+        <v>641</v>
+      </c>
+      <c r="E298" s="1" t="n">
+        <v>46153.50941356482</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>238</v>
+      </c>
+      <c r="C299" t="n">
+        <v>0</v>
+      </c>
+      <c r="D299" t="n">
+        <v>915</v>
+      </c>
+      <c r="E299" s="1" t="n">
+        <v>46153.50941356482</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>245</v>
+      </c>
+      <c r="C300" t="n">
+        <v>0</v>
+      </c>
+      <c r="D300" t="n">
+        <v>87</v>
+      </c>
+      <c r="E300" s="1" t="n">
+        <v>46153.65715731774</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>0</v>
+      </c>
+      <c r="C301" t="n">
+        <v>0</v>
+      </c>
+      <c r="D301" t="n">
+        <v>87</v>
+      </c>
+      <c r="E301" s="1" t="n">
+        <v>46153.65715731774</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>0</v>
+      </c>
+      <c r="C302" t="n">
+        <v>0</v>
+      </c>
+      <c r="D302" t="n">
+        <v>87</v>
+      </c>
+      <c r="E302" s="1" t="n">
+        <v>46153.65715731774</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>0</v>
+      </c>
+      <c r="C303" t="n">
+        <v>0</v>
+      </c>
+      <c r="D303" t="n">
+        <v>87</v>
+      </c>
+      <c r="E303" s="1" t="n">
+        <v>46153.65715731774</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>0</v>
+      </c>
+      <c r="C304" t="n">
+        <v>0</v>
+      </c>
+      <c r="D304" t="n">
+        <v>87</v>
+      </c>
+      <c r="E304" s="1" t="n">
+        <v>46153.65715731774</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizações de formatação e correção na saída da coluna Valor total
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E304"/>
+  <dimension ref="A1:E329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6125,7 +6125,7 @@
         <v>87</v>
       </c>
       <c r="E300" s="1" t="n">
-        <v>46153.65715731774</v>
+        <v>46153.65715731482</v>
       </c>
     </row>
     <row r="301">
@@ -6144,7 +6144,7 @@
         <v>87</v>
       </c>
       <c r="E301" s="1" t="n">
-        <v>46153.65715731774</v>
+        <v>46153.65715731482</v>
       </c>
     </row>
     <row r="302">
@@ -6163,7 +6163,7 @@
         <v>87</v>
       </c>
       <c r="E302" s="1" t="n">
-        <v>46153.65715731774</v>
+        <v>46153.65715731482</v>
       </c>
     </row>
     <row r="303">
@@ -6182,7 +6182,7 @@
         <v>87</v>
       </c>
       <c r="E303" s="1" t="n">
-        <v>46153.65715731774</v>
+        <v>46153.65715731482</v>
       </c>
     </row>
     <row r="304">
@@ -6201,7 +6201,482 @@
         <v>87</v>
       </c>
       <c r="E304" s="1" t="n">
-        <v>46153.65715731774</v>
+        <v>46153.65715731482</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>245</v>
+      </c>
+      <c r="C305" t="n">
+        <v>0</v>
+      </c>
+      <c r="D305" t="n">
+        <v>87</v>
+      </c>
+      <c r="E305" s="1" t="n">
+        <v>46153.69541155093</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>0</v>
+      </c>
+      <c r="C306" t="n">
+        <v>0</v>
+      </c>
+      <c r="D306" t="n">
+        <v>87</v>
+      </c>
+      <c r="E306" s="1" t="n">
+        <v>46153.69541155093</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>0</v>
+      </c>
+      <c r="C307" t="n">
+        <v>0</v>
+      </c>
+      <c r="D307" t="n">
+        <v>87</v>
+      </c>
+      <c r="E307" s="1" t="n">
+        <v>46153.69541155093</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>0</v>
+      </c>
+      <c r="C308" t="n">
+        <v>0</v>
+      </c>
+      <c r="D308" t="n">
+        <v>87</v>
+      </c>
+      <c r="E308" s="1" t="n">
+        <v>46153.69541155093</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>0</v>
+      </c>
+      <c r="C309" t="n">
+        <v>0</v>
+      </c>
+      <c r="D309" t="n">
+        <v>87</v>
+      </c>
+      <c r="E309" s="1" t="n">
+        <v>46153.69541155093</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C310" t="n">
+        <v>0</v>
+      </c>
+      <c r="D310" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E310" s="1" t="n">
+        <v>46153.69686677084</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>0</v>
+      </c>
+      <c r="C311" t="n">
+        <v>0</v>
+      </c>
+      <c r="D311" t="n">
+        <v>641</v>
+      </c>
+      <c r="E311" s="1" t="n">
+        <v>46153.69686677084</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>67</v>
+      </c>
+      <c r="C312" t="n">
+        <v>0</v>
+      </c>
+      <c r="D312" t="n">
+        <v>574</v>
+      </c>
+      <c r="E312" s="1" t="n">
+        <v>46153.69686677084</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>274</v>
+      </c>
+      <c r="C313" t="n">
+        <v>0</v>
+      </c>
+      <c r="D313" t="n">
+        <v>641</v>
+      </c>
+      <c r="E313" s="1" t="n">
+        <v>46153.69686677084</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>238</v>
+      </c>
+      <c r="C314" t="n">
+        <v>0</v>
+      </c>
+      <c r="D314" t="n">
+        <v>915</v>
+      </c>
+      <c r="E314" s="1" t="n">
+        <v>46153.69686677084</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C315" t="n">
+        <v>0</v>
+      </c>
+      <c r="D315" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E315" s="1" t="n">
+        <v>46153.75516246528</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>0</v>
+      </c>
+      <c r="C316" t="n">
+        <v>0</v>
+      </c>
+      <c r="D316" t="n">
+        <v>641</v>
+      </c>
+      <c r="E316" s="1" t="n">
+        <v>46153.75516246528</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>67</v>
+      </c>
+      <c r="C317" t="n">
+        <v>0</v>
+      </c>
+      <c r="D317" t="n">
+        <v>574</v>
+      </c>
+      <c r="E317" s="1" t="n">
+        <v>46153.75516246528</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>274</v>
+      </c>
+      <c r="C318" t="n">
+        <v>0</v>
+      </c>
+      <c r="D318" t="n">
+        <v>641</v>
+      </c>
+      <c r="E318" s="1" t="n">
+        <v>46153.75516246528</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B319" t="n">
+        <v>238</v>
+      </c>
+      <c r="C319" t="n">
+        <v>0</v>
+      </c>
+      <c r="D319" t="n">
+        <v>915</v>
+      </c>
+      <c r="E319" s="1" t="n">
+        <v>46153.75516246528</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B320" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C320" t="n">
+        <v>0</v>
+      </c>
+      <c r="D320" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E320" s="1" t="n">
+        <v>46153.75769523148</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>0</v>
+      </c>
+      <c r="C321" t="n">
+        <v>0</v>
+      </c>
+      <c r="D321" t="n">
+        <v>641</v>
+      </c>
+      <c r="E321" s="1" t="n">
+        <v>46153.75769523148</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>67</v>
+      </c>
+      <c r="C322" t="n">
+        <v>0</v>
+      </c>
+      <c r="D322" t="n">
+        <v>574</v>
+      </c>
+      <c r="E322" s="1" t="n">
+        <v>46153.75769523148</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>274</v>
+      </c>
+      <c r="C323" t="n">
+        <v>0</v>
+      </c>
+      <c r="D323" t="n">
+        <v>641</v>
+      </c>
+      <c r="E323" s="1" t="n">
+        <v>46153.75769523148</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B324" t="n">
+        <v>238</v>
+      </c>
+      <c r="C324" t="n">
+        <v>0</v>
+      </c>
+      <c r="D324" t="n">
+        <v>915</v>
+      </c>
+      <c r="E324" s="1" t="n">
+        <v>46153.75769523148</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B325" t="n">
+        <v>1511</v>
+      </c>
+      <c r="C325" t="n">
+        <v>0</v>
+      </c>
+      <c r="D325" t="n">
+        <v>1153</v>
+      </c>
+      <c r="E325" s="1" t="n">
+        <v>46153.76245916515</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B326" t="n">
+        <v>0</v>
+      </c>
+      <c r="C326" t="n">
+        <v>0</v>
+      </c>
+      <c r="D326" t="n">
+        <v>641</v>
+      </c>
+      <c r="E326" s="1" t="n">
+        <v>46153.76245916515</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>67</v>
+      </c>
+      <c r="C327" t="n">
+        <v>0</v>
+      </c>
+      <c r="D327" t="n">
+        <v>574</v>
+      </c>
+      <c r="E327" s="1" t="n">
+        <v>46153.76245916515</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>274</v>
+      </c>
+      <c r="C328" t="n">
+        <v>0</v>
+      </c>
+      <c r="D328" t="n">
+        <v>641</v>
+      </c>
+      <c r="E328" s="1" t="n">
+        <v>46153.76245916515</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B329" t="n">
+        <v>238</v>
+      </c>
+      <c r="C329" t="n">
+        <v>0</v>
+      </c>
+      <c r="D329" t="n">
+        <v>915</v>
+      </c>
+      <c r="E329" s="1" t="n">
+        <v>46153.76245916515</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Ajuste na lógica de exportação para o email
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E329"/>
+  <dimension ref="A1:E349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6600,7 +6600,7 @@
         <v>1153</v>
       </c>
       <c r="E325" s="1" t="n">
-        <v>46153.76245916515</v>
+        <v>46153.76245916667</v>
       </c>
     </row>
     <row r="326">
@@ -6619,7 +6619,7 @@
         <v>641</v>
       </c>
       <c r="E326" s="1" t="n">
-        <v>46153.76245916515</v>
+        <v>46153.76245916667</v>
       </c>
     </row>
     <row r="327">
@@ -6638,7 +6638,7 @@
         <v>574</v>
       </c>
       <c r="E327" s="1" t="n">
-        <v>46153.76245916515</v>
+        <v>46153.76245916667</v>
       </c>
     </row>
     <row r="328">
@@ -6657,7 +6657,7 @@
         <v>641</v>
       </c>
       <c r="E328" s="1" t="n">
-        <v>46153.76245916515</v>
+        <v>46153.76245916667</v>
       </c>
     </row>
     <row r="329">
@@ -6676,7 +6676,387 @@
         <v>915</v>
       </c>
       <c r="E329" s="1" t="n">
-        <v>46153.76245916515</v>
+        <v>46153.76245916667</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B330" t="n">
+        <v>1512</v>
+      </c>
+      <c r="C330" t="n">
+        <v>0</v>
+      </c>
+      <c r="D330" t="n">
+        <v>1152</v>
+      </c>
+      <c r="E330" s="1" t="n">
+        <v>46154.40578791666</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>0</v>
+      </c>
+      <c r="C331" t="n">
+        <v>0</v>
+      </c>
+      <c r="D331" t="n">
+        <v>636</v>
+      </c>
+      <c r="E331" s="1" t="n">
+        <v>46154.40578791666</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B332" t="n">
+        <v>64</v>
+      </c>
+      <c r="C332" t="n">
+        <v>0</v>
+      </c>
+      <c r="D332" t="n">
+        <v>572</v>
+      </c>
+      <c r="E332" s="1" t="n">
+        <v>46154.40578791666</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B333" t="n">
+        <v>278</v>
+      </c>
+      <c r="C333" t="n">
+        <v>0</v>
+      </c>
+      <c r="D333" t="n">
+        <v>636</v>
+      </c>
+      <c r="E333" s="1" t="n">
+        <v>46154.40578791666</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B334" t="n">
+        <v>238</v>
+      </c>
+      <c r="C334" t="n">
+        <v>0</v>
+      </c>
+      <c r="D334" t="n">
+        <v>914</v>
+      </c>
+      <c r="E334" s="1" t="n">
+        <v>46154.40578791666</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B335" t="n">
+        <v>1512</v>
+      </c>
+      <c r="C335" t="n">
+        <v>0</v>
+      </c>
+      <c r="D335" t="n">
+        <v>1152</v>
+      </c>
+      <c r="E335" s="1" t="n">
+        <v>46154.40791271991</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B336" t="n">
+        <v>0</v>
+      </c>
+      <c r="C336" t="n">
+        <v>0</v>
+      </c>
+      <c r="D336" t="n">
+        <v>636</v>
+      </c>
+      <c r="E336" s="1" t="n">
+        <v>46154.40791271991</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B337" t="n">
+        <v>64</v>
+      </c>
+      <c r="C337" t="n">
+        <v>0</v>
+      </c>
+      <c r="D337" t="n">
+        <v>572</v>
+      </c>
+      <c r="E337" s="1" t="n">
+        <v>46154.40791271991</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B338" t="n">
+        <v>278</v>
+      </c>
+      <c r="C338" t="n">
+        <v>0</v>
+      </c>
+      <c r="D338" t="n">
+        <v>636</v>
+      </c>
+      <c r="E338" s="1" t="n">
+        <v>46154.40791271991</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>238</v>
+      </c>
+      <c r="C339" t="n">
+        <v>0</v>
+      </c>
+      <c r="D339" t="n">
+        <v>914</v>
+      </c>
+      <c r="E339" s="1" t="n">
+        <v>46154.40791271991</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B340" t="n">
+        <v>245</v>
+      </c>
+      <c r="C340" t="n">
+        <v>0</v>
+      </c>
+      <c r="D340" t="n">
+        <v>87</v>
+      </c>
+      <c r="E340" s="1" t="n">
+        <v>46154.42793541666</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B341" t="n">
+        <v>0</v>
+      </c>
+      <c r="C341" t="n">
+        <v>0</v>
+      </c>
+      <c r="D341" t="n">
+        <v>87</v>
+      </c>
+      <c r="E341" s="1" t="n">
+        <v>46154.42793541666</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B342" t="n">
+        <v>0</v>
+      </c>
+      <c r="C342" t="n">
+        <v>0</v>
+      </c>
+      <c r="D342" t="n">
+        <v>87</v>
+      </c>
+      <c r="E342" s="1" t="n">
+        <v>46154.42793541666</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B343" t="n">
+        <v>0</v>
+      </c>
+      <c r="C343" t="n">
+        <v>0</v>
+      </c>
+      <c r="D343" t="n">
+        <v>87</v>
+      </c>
+      <c r="E343" s="1" t="n">
+        <v>46154.42793541666</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B344" t="n">
+        <v>0</v>
+      </c>
+      <c r="C344" t="n">
+        <v>0</v>
+      </c>
+      <c r="D344" t="n">
+        <v>87</v>
+      </c>
+      <c r="E344" s="1" t="n">
+        <v>46154.42793541666</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>1512</v>
+      </c>
+      <c r="C345" t="n">
+        <v>0</v>
+      </c>
+      <c r="D345" t="n">
+        <v>1152</v>
+      </c>
+      <c r="E345" s="1" t="n">
+        <v>46154.43059595256</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B346" t="n">
+        <v>0</v>
+      </c>
+      <c r="C346" t="n">
+        <v>0</v>
+      </c>
+      <c r="D346" t="n">
+        <v>636</v>
+      </c>
+      <c r="E346" s="1" t="n">
+        <v>46154.43059595256</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B347" t="n">
+        <v>64</v>
+      </c>
+      <c r="C347" t="n">
+        <v>0</v>
+      </c>
+      <c r="D347" t="n">
+        <v>572</v>
+      </c>
+      <c r="E347" s="1" t="n">
+        <v>46154.43059595256</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B348" t="n">
+        <v>278</v>
+      </c>
+      <c r="C348" t="n">
+        <v>0</v>
+      </c>
+      <c r="D348" t="n">
+        <v>636</v>
+      </c>
+      <c r="E348" s="1" t="n">
+        <v>46154.43059595256</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B349" t="n">
+        <v>238</v>
+      </c>
+      <c r="C349" t="n">
+        <v>0</v>
+      </c>
+      <c r="D349" t="n">
+        <v>914</v>
+      </c>
+      <c r="E349" s="1" t="n">
+        <v>46154.43059595256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: inclusão de nova coluna no log detalhado informando qual foi o usuário que executou a rotina
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -463,7 +463,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46154.52336809108</v>
+        <v>46154.54932493867</v>
       </c>
     </row>
     <row r="3">
@@ -482,7 +482,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>46154.52336809108</v>
+        <v>46154.54932493867</v>
       </c>
     </row>
     <row r="4">
@@ -501,7 +501,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>46154.52336809108</v>
+        <v>46154.54932493867</v>
       </c>
     </row>
     <row r="5">
@@ -520,7 +520,7 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>46154.52336809108</v>
+        <v>46154.54932493867</v>
       </c>
     </row>
     <row r="6">
@@ -539,7 +539,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>46154.52336809108</v>
+        <v>46154.54932493867</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajustes feitos: ' Ajutes no flag de email que estava desmarcando ao avançar na segunda etapa do menu ' correção na duplicidade de textos após um erro mapeado ' correção no relógio de carregamento apresentado no final do processamento ' inclusão de popup para confirmar se deseja enviar ou não o email
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="E87" s="1" t="n">
-        <v>46155.71885253557</v>
+        <v>46155.71885253472</v>
       </c>
     </row>
     <row r="88">
@@ -2097,7 +2097,7 @@
         <v>0</v>
       </c>
       <c r="E88" s="1" t="n">
-        <v>46155.71885253557</v>
+        <v>46155.71885253472</v>
       </c>
     </row>
     <row r="89">
@@ -2116,7 +2116,7 @@
         <v>0</v>
       </c>
       <c r="E89" s="1" t="n">
-        <v>46155.71885253557</v>
+        <v>46155.71885253472</v>
       </c>
     </row>
     <row r="90">
@@ -2135,7 +2135,7 @@
         <v>0</v>
       </c>
       <c r="E90" s="1" t="n">
-        <v>46155.71885253557</v>
+        <v>46155.71885253472</v>
       </c>
     </row>
     <row r="91">
@@ -2154,7 +2154,292 @@
         <v>0</v>
       </c>
       <c r="E91" s="1" t="n">
-        <v>46155.71885253557</v>
+        <v>46155.71885253472</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1304</v>
+      </c>
+      <c r="C92" t="n">
+        <v>1310</v>
+      </c>
+      <c r="D92" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" s="1" t="n">
+        <v>46156.46741908565</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0</v>
+      </c>
+      <c r="C93" t="n">
+        <v>751</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" s="1" t="n">
+        <v>46156.46741908565</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>20</v>
+      </c>
+      <c r="C94" t="n">
+        <v>731</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" s="1" t="n">
+        <v>46156.46741908565</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>360</v>
+      </c>
+      <c r="C95" t="n">
+        <v>751</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="1" t="n">
+        <v>46156.46741908565</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>199</v>
+      </c>
+      <c r="C96" t="n">
+        <v>1111</v>
+      </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="1" t="n">
+        <v>46156.46741908565</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>1304</v>
+      </c>
+      <c r="C97" t="n">
+        <v>1310</v>
+      </c>
+      <c r="D97" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="1" t="n">
+        <v>46156.46883369213</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" t="n">
+        <v>751</v>
+      </c>
+      <c r="D98" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" s="1" t="n">
+        <v>46156.46883369213</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>20</v>
+      </c>
+      <c r="C99" t="n">
+        <v>731</v>
+      </c>
+      <c r="D99" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="1" t="n">
+        <v>46156.46883369213</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>360</v>
+      </c>
+      <c r="C100" t="n">
+        <v>751</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="1" t="n">
+        <v>46156.46883369213</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>199</v>
+      </c>
+      <c r="C101" t="n">
+        <v>1111</v>
+      </c>
+      <c r="D101" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="1" t="n">
+        <v>46156.46883369213</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1304</v>
+      </c>
+      <c r="C102" t="n">
+        <v>1310</v>
+      </c>
+      <c r="D102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="1" t="n">
+        <v>46156.47054966824</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>0</v>
+      </c>
+      <c r="C103" t="n">
+        <v>751</v>
+      </c>
+      <c r="D103" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" s="1" t="n">
+        <v>46156.47054966824</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>20</v>
+      </c>
+      <c r="C104" t="n">
+        <v>731</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" s="1" t="n">
+        <v>46156.47054966824</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>360</v>
+      </c>
+      <c r="C105" t="n">
+        <v>751</v>
+      </c>
+      <c r="D105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="1" t="n">
+        <v>46156.47054966824</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>199</v>
+      </c>
+      <c r="C106" t="n">
+        <v>1111</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" s="1" t="n">
+        <v>46156.47054966824</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat:                                        ' Ajustes no log, alterando seu tipo de incrementação + envio de email unico por celula e email geral para gestão
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,16 +454,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1512</v>
+        <v>1307</v>
       </c>
       <c r="C2" t="n">
-        <v>1152</v>
+        <v>1307</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46154.54932494213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="3">
@@ -476,13 +476,13 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>636</v>
+        <v>745</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>46154.54932494213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="4">
@@ -492,16 +492,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C4" t="n">
-        <v>572</v>
+        <v>724</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>46154.54932494213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="5">
@@ -511,16 +511,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C5" t="n">
-        <v>636</v>
+        <v>745</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>46154.54932494213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="6">
@@ -530,16 +530,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C6" t="n">
-        <v>914</v>
+        <v>1108</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>46154.54932494213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="7">
@@ -549,16 +549,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1512</v>
+        <v>1307</v>
       </c>
       <c r="C7" t="n">
-        <v>1152</v>
+        <v>1307</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>46154.65916084491</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="8">
@@ -571,13 +571,13 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>636</v>
+        <v>745</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>46154.65916084491</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="9">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C9" t="n">
-        <v>572</v>
+        <v>724</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>46154.65916084491</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="10">
@@ -606,16 +606,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C10" t="n">
-        <v>636</v>
+        <v>745</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>46154.65916084491</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="11">
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C11" t="n">
-        <v>914</v>
+        <v>1108</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>46154.65916084491</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="12">
@@ -644,16 +644,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C12" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>46155.46399839121</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="13">
@@ -666,13 +666,13 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>46155.46399839121</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="14">
@@ -682,16 +682,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C14" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>46155.46399839121</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="15">
@@ -701,16 +701,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C15" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>46155.46399839121</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="16">
@@ -720,16 +720,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C16" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>46155.46399839121</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="17">
@@ -739,16 +739,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C17" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>46155.47890324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="18">
@@ -761,13 +761,13 @@
         <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>46155.47890324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="19">
@@ -777,16 +777,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C19" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>46155.47890324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="20">
@@ -796,16 +796,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C20" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>46155.47890324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="21">
@@ -815,16 +815,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C21" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>46155.47890324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="22">
@@ -834,16 +834,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C22" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>46155.48085587963</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="23">
@@ -856,13 +856,13 @@
         <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="1" t="n">
-        <v>46155.48085587963</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="24">
@@ -872,16 +872,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C24" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="1" t="n">
-        <v>46155.48085587963</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="25">
@@ -891,16 +891,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C25" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>46155.48085587963</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="26">
@@ -910,16 +910,16 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C26" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="1" t="n">
-        <v>46155.48085587963</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="27">
@@ -929,16 +929,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C27" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="1" t="n">
-        <v>46155.48230046297</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="28">
@@ -951,13 +951,13 @@
         <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="1" t="n">
-        <v>46155.48230046297</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="29">
@@ -967,16 +967,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C29" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="1" t="n">
-        <v>46155.48230046297</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="30">
@@ -986,16 +986,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C30" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="1" t="n">
-        <v>46155.48230046297</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="31">
@@ -1005,16 +1005,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C31" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="1" t="n">
-        <v>46155.48230046297</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="32">
@@ -1024,16 +1024,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C32" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="1" t="n">
-        <v>46155.49551653935</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="33">
@@ -1046,13 +1046,13 @@
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
       <c r="E33" s="1" t="n">
-        <v>46155.49551653935</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="34">
@@ -1062,16 +1062,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C34" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="1" t="n">
-        <v>46155.49551653935</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="35">
@@ -1081,16 +1081,16 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C35" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="1" t="n">
-        <v>46155.49551653935</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="36">
@@ -1100,16 +1100,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C36" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="1" t="n">
-        <v>46155.49551653935</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="37">
@@ -1119,16 +1119,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C37" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="1" t="n">
-        <v>46155.50603189815</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="38">
@@ -1141,13 +1141,13 @@
         <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
       <c r="E38" s="1" t="n">
-        <v>46155.50603189815</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="39">
@@ -1157,16 +1157,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C39" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
       </c>
       <c r="E39" s="1" t="n">
-        <v>46155.50603189815</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="40">
@@ -1176,16 +1176,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C40" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
       </c>
       <c r="E40" s="1" t="n">
-        <v>46155.50603189815</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="41">
@@ -1195,16 +1195,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C41" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
       </c>
       <c r="E41" s="1" t="n">
-        <v>46155.50603189815</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="42">
@@ -1214,16 +1214,16 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C42" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="1" t="n">
-        <v>46155.5097794213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="43">
@@ -1236,13 +1236,13 @@
         <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="1" t="n">
-        <v>46155.5097794213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="44">
@@ -1252,16 +1252,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C44" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
       </c>
       <c r="E44" s="1" t="n">
-        <v>46155.5097794213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="45">
@@ -1271,16 +1271,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C45" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
       </c>
       <c r="E45" s="1" t="n">
-        <v>46155.5097794213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="46">
@@ -1290,16 +1290,16 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C46" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D46" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="1" t="n">
-        <v>46155.5097794213</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="47">
@@ -1309,16 +1309,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C47" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="1" t="n">
-        <v>46155.51135291667</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="48">
@@ -1331,13 +1331,13 @@
         <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
       </c>
       <c r="E48" s="1" t="n">
-        <v>46155.51135291667</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="49">
@@ -1347,16 +1347,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C49" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
       </c>
       <c r="E49" s="1" t="n">
-        <v>46155.51135291667</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="50">
@@ -1366,16 +1366,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C50" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
       </c>
       <c r="E50" s="1" t="n">
-        <v>46155.51135291667</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="51">
@@ -1385,16 +1385,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C51" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
       </c>
       <c r="E51" s="1" t="n">
-        <v>46155.51135291667</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="52">
@@ -1404,16 +1404,16 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C52" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
       </c>
       <c r="E52" s="1" t="n">
-        <v>46155.51683324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="53">
@@ -1426,13 +1426,13 @@
         <v>0</v>
       </c>
       <c r="C53" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
       </c>
       <c r="E53" s="1" t="n">
-        <v>46155.51683324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="54">
@@ -1442,16 +1442,16 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C54" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="1" t="n">
-        <v>46155.51683324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="55">
@@ -1461,16 +1461,16 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C55" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
       </c>
       <c r="E55" s="1" t="n">
-        <v>46155.51683324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="56">
@@ -1480,16 +1480,16 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C56" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
       </c>
       <c r="E56" s="1" t="n">
-        <v>46155.51683324074</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="57">
@@ -1499,16 +1499,16 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C57" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
       </c>
       <c r="E57" s="1" t="n">
-        <v>46155.52703618055</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="58">
@@ -1521,13 +1521,13 @@
         <v>0</v>
       </c>
       <c r="C58" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
       </c>
       <c r="E58" s="1" t="n">
-        <v>46155.52703618055</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="59">
@@ -1537,16 +1537,16 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C59" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
       </c>
       <c r="E59" s="1" t="n">
-        <v>46155.52703618055</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="60">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C60" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
       </c>
       <c r="E60" s="1" t="n">
-        <v>46155.52703618055</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="61">
@@ -1575,16 +1575,16 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C61" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
       </c>
       <c r="E61" s="1" t="n">
-        <v>46155.52703618055</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="62">
@@ -1594,16 +1594,16 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C62" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
       </c>
       <c r="E62" s="1" t="n">
-        <v>46155.53353721065</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="63">
@@ -1616,13 +1616,13 @@
         <v>0</v>
       </c>
       <c r="C63" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
       </c>
       <c r="E63" s="1" t="n">
-        <v>46155.53353721065</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="64">
@@ -1632,16 +1632,16 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C64" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
       </c>
       <c r="E64" s="1" t="n">
-        <v>46155.53353721065</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="65">
@@ -1651,16 +1651,16 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C65" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
       </c>
       <c r="E65" s="1" t="n">
-        <v>46155.53353721065</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="66">
@@ -1670,16 +1670,16 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C66" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>
       </c>
       <c r="E66" s="1" t="n">
-        <v>46155.53353721065</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="67">
@@ -1689,16 +1689,16 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C67" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D67" t="n">
         <v>0</v>
       </c>
       <c r="E67" s="1" t="n">
-        <v>46155.53534734953</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="68">
@@ -1711,13 +1711,13 @@
         <v>0</v>
       </c>
       <c r="C68" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D68" t="n">
         <v>0</v>
       </c>
       <c r="E68" s="1" t="n">
-        <v>46155.53534734953</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="69">
@@ -1727,16 +1727,16 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C69" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
       </c>
       <c r="E69" s="1" t="n">
-        <v>46155.53534734953</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="70">
@@ -1746,16 +1746,16 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C70" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D70" t="n">
         <v>0</v>
       </c>
       <c r="E70" s="1" t="n">
-        <v>46155.53534734953</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="71">
@@ -1765,16 +1765,16 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C71" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D71" t="n">
         <v>0</v>
       </c>
       <c r="E71" s="1" t="n">
-        <v>46155.53534734953</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="72">
@@ -1784,16 +1784,16 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C72" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D72" t="n">
         <v>0</v>
       </c>
       <c r="E72" s="1" t="n">
-        <v>46155.63263775463</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="73">
@@ -1806,13 +1806,13 @@
         <v>0</v>
       </c>
       <c r="C73" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D73" t="n">
         <v>0</v>
       </c>
       <c r="E73" s="1" t="n">
-        <v>46155.63263775463</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="74">
@@ -1822,16 +1822,16 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C74" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D74" t="n">
         <v>0</v>
       </c>
       <c r="E74" s="1" t="n">
-        <v>46155.63263775463</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="75">
@@ -1841,16 +1841,16 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C75" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D75" t="n">
         <v>0</v>
       </c>
       <c r="E75" s="1" t="n">
-        <v>46155.63263775463</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="76">
@@ -1860,16 +1860,16 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C76" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D76" t="n">
         <v>0</v>
       </c>
       <c r="E76" s="1" t="n">
-        <v>46155.63263775463</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="77">
@@ -1879,16 +1879,16 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1513</v>
+        <v>1307</v>
       </c>
       <c r="C77" t="n">
-        <v>1151</v>
+        <v>1307</v>
       </c>
       <c r="D77" t="n">
         <v>0</v>
       </c>
       <c r="E77" s="1" t="n">
-        <v>46155.70339077546</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="78">
@@ -1901,13 +1901,13 @@
         <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
       </c>
       <c r="E78" s="1" t="n">
-        <v>46155.70339077546</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="79">
@@ -1917,16 +1917,16 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C79" t="n">
-        <v>571</v>
+        <v>724</v>
       </c>
       <c r="D79" t="n">
         <v>0</v>
       </c>
       <c r="E79" s="1" t="n">
-        <v>46155.70339077546</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="80">
@@ -1936,16 +1936,16 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>278</v>
+        <v>363</v>
       </c>
       <c r="C80" t="n">
-        <v>635</v>
+        <v>745</v>
       </c>
       <c r="D80" t="n">
         <v>0</v>
       </c>
       <c r="E80" s="1" t="n">
-        <v>46155.70339077546</v>
+        <v>46157</v>
       </c>
     </row>
     <row r="81">
@@ -1955,491 +1955,16 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>238</v>
+        <v>199</v>
       </c>
       <c r="C81" t="n">
-        <v>913</v>
+        <v>1108</v>
       </c>
       <c r="D81" t="n">
         <v>0</v>
       </c>
       <c r="E81" s="1" t="n">
-        <v>46155.70339077546</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Chave Aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>1513</v>
-      </c>
-      <c r="C82" t="n">
-        <v>1151</v>
-      </c>
-      <c r="D82" t="n">
-        <v>0</v>
-      </c>
-      <c r="E82" s="1" t="n">
-        <v>46155.71229060185</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Data + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>0</v>
-      </c>
-      <c r="C83" t="n">
-        <v>635</v>
-      </c>
-      <c r="D83" t="n">
-        <v>0</v>
-      </c>
-      <c r="E83" s="1" t="n">
-        <v>46155.71229060185</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>64</v>
-      </c>
-      <c r="C84" t="n">
-        <v>571</v>
-      </c>
-      <c r="D84" t="n">
-        <v>0</v>
-      </c>
-      <c r="E84" s="1" t="n">
-        <v>46155.71229060185</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>Chave Loc Cia + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B85" t="n">
-        <v>278</v>
-      </c>
-      <c r="C85" t="n">
-        <v>635</v>
-      </c>
-      <c r="D85" t="n">
-        <v>0</v>
-      </c>
-      <c r="E85" s="1" t="n">
-        <v>46155.71229060185</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Chave nr_aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B86" t="n">
-        <v>238</v>
-      </c>
-      <c r="C86" t="n">
-        <v>913</v>
-      </c>
-      <c r="D86" t="n">
-        <v>0</v>
-      </c>
-      <c r="E86" s="1" t="n">
-        <v>46155.71229060185</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>Chave Aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B87" t="n">
-        <v>1298</v>
-      </c>
-      <c r="C87" t="n">
-        <v>1316</v>
-      </c>
-      <c r="D87" t="n">
-        <v>0</v>
-      </c>
-      <c r="E87" s="1" t="n">
-        <v>46155.71885253472</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Data + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B88" t="n">
-        <v>0</v>
-      </c>
-      <c r="C88" t="n">
-        <v>763</v>
-      </c>
-      <c r="D88" t="n">
-        <v>0</v>
-      </c>
-      <c r="E88" s="1" t="n">
-        <v>46155.71885253472</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B89" t="n">
-        <v>20</v>
-      </c>
-      <c r="C89" t="n">
-        <v>743</v>
-      </c>
-      <c r="D89" t="n">
-        <v>0</v>
-      </c>
-      <c r="E89" s="1" t="n">
-        <v>46155.71885253472</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>Chave Loc Cia + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B90" t="n">
-        <v>358</v>
-      </c>
-      <c r="C90" t="n">
-        <v>763</v>
-      </c>
-      <c r="D90" t="n">
-        <v>0</v>
-      </c>
-      <c r="E90" s="1" t="n">
-        <v>46155.71885253472</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>Chave nr_aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B91" t="n">
-        <v>195</v>
-      </c>
-      <c r="C91" t="n">
-        <v>1121</v>
-      </c>
-      <c r="D91" t="n">
-        <v>0</v>
-      </c>
-      <c r="E91" s="1" t="n">
-        <v>46155.71885253472</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>Chave Aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B92" t="n">
-        <v>1304</v>
-      </c>
-      <c r="C92" t="n">
-        <v>1310</v>
-      </c>
-      <c r="D92" t="n">
-        <v>0</v>
-      </c>
-      <c r="E92" s="1" t="n">
-        <v>46156.46741908565</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Data + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
-        <v>0</v>
-      </c>
-      <c r="C93" t="n">
-        <v>751</v>
-      </c>
-      <c r="D93" t="n">
-        <v>0</v>
-      </c>
-      <c r="E93" s="1" t="n">
-        <v>46156.46741908565</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
-        <v>20</v>
-      </c>
-      <c r="C94" t="n">
-        <v>731</v>
-      </c>
-      <c r="D94" t="n">
-        <v>0</v>
-      </c>
-      <c r="E94" s="1" t="n">
-        <v>46156.46741908565</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Chave Loc Cia + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B95" t="n">
-        <v>360</v>
-      </c>
-      <c r="C95" t="n">
-        <v>751</v>
-      </c>
-      <c r="D95" t="n">
-        <v>0</v>
-      </c>
-      <c r="E95" s="1" t="n">
-        <v>46156.46741908565</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>Chave nr_aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B96" t="n">
-        <v>199</v>
-      </c>
-      <c r="C96" t="n">
-        <v>1111</v>
-      </c>
-      <c r="D96" t="n">
-        <v>0</v>
-      </c>
-      <c r="E96" s="1" t="n">
-        <v>46156.46741908565</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Chave Aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B97" t="n">
-        <v>1304</v>
-      </c>
-      <c r="C97" t="n">
-        <v>1310</v>
-      </c>
-      <c r="D97" t="n">
-        <v>0</v>
-      </c>
-      <c r="E97" s="1" t="n">
-        <v>46156.46883369213</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Data + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B98" t="n">
-        <v>0</v>
-      </c>
-      <c r="C98" t="n">
-        <v>751</v>
-      </c>
-      <c r="D98" t="n">
-        <v>0</v>
-      </c>
-      <c r="E98" s="1" t="n">
-        <v>46156.46883369213</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B99" t="n">
-        <v>20</v>
-      </c>
-      <c r="C99" t="n">
-        <v>731</v>
-      </c>
-      <c r="D99" t="n">
-        <v>0</v>
-      </c>
-      <c r="E99" s="1" t="n">
-        <v>46156.46883369213</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Chave Loc Cia + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B100" t="n">
-        <v>360</v>
-      </c>
-      <c r="C100" t="n">
-        <v>751</v>
-      </c>
-      <c r="D100" t="n">
-        <v>0</v>
-      </c>
-      <c r="E100" s="1" t="n">
-        <v>46156.46883369213</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>Chave nr_aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B101" t="n">
-        <v>199</v>
-      </c>
-      <c r="C101" t="n">
-        <v>1111</v>
-      </c>
-      <c r="D101" t="n">
-        <v>0</v>
-      </c>
-      <c r="E101" s="1" t="n">
-        <v>46156.46883369213</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Chave Aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B102" t="n">
-        <v>1304</v>
-      </c>
-      <c r="C102" t="n">
-        <v>1310</v>
-      </c>
-      <c r="D102" t="n">
-        <v>0</v>
-      </c>
-      <c r="E102" s="1" t="n">
-        <v>46156.47054966824</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Data + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B103" t="n">
-        <v>0</v>
-      </c>
-      <c r="C103" t="n">
-        <v>751</v>
-      </c>
-      <c r="D103" t="n">
-        <v>0</v>
-      </c>
-      <c r="E103" s="1" t="n">
-        <v>46156.47054966824</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>Chave Cartão + Valor + Loc Cia</t>
-        </is>
-      </c>
-      <c r="B104" t="n">
-        <v>20</v>
-      </c>
-      <c r="C104" t="n">
-        <v>731</v>
-      </c>
-      <c r="D104" t="n">
-        <v>0</v>
-      </c>
-      <c r="E104" s="1" t="n">
-        <v>46156.47054966824</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>Chave Loc Cia + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B105" t="n">
-        <v>360</v>
-      </c>
-      <c r="C105" t="n">
-        <v>751</v>
-      </c>
-      <c r="D105" t="n">
-        <v>0</v>
-      </c>
-      <c r="E105" s="1" t="n">
-        <v>46156.47054966824</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Chave nr_aut + Data + Valor</t>
-        </is>
-      </c>
-      <c r="B106" t="n">
-        <v>199</v>
-      </c>
-      <c r="C106" t="n">
-        <v>1111</v>
-      </c>
-      <c r="D106" t="n">
-        <v>0</v>
-      </c>
-      <c r="E106" s="1" t="n">
-        <v>46156.47054966824</v>
+        <v>46157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Ajuste no escopo dos emails e lógica de envio
</commit_message>
<xml_diff>
--- a/logs/historico_execucao.xlsx
+++ b/logs/historico_execucao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2157,6 +2157,101 @@
         <v>46161</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Chave Aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1580</v>
+      </c>
+      <c r="C92" t="n">
+        <v>1585</v>
+      </c>
+      <c r="D92" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" s="1" t="n">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Data + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0</v>
+      </c>
+      <c r="C93" t="n">
+        <v>912</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" s="1" t="n">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Chave Cartão + Valor + Loc Cia</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>25</v>
+      </c>
+      <c r="C94" t="n">
+        <v>887</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" s="1" t="n">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Chave Loc Cia + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>422</v>
+      </c>
+      <c r="C95" t="n">
+        <v>912</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="1" t="n">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Chave nr_aut + Data + Valor</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>251</v>
+      </c>
+      <c r="C96" t="n">
+        <v>1334</v>
+      </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="1" t="n">
+        <v>46163</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>